<commit_message>
Expand Evergreen Dev Co from 3 to 11 projects in Current_Projects sheet
https://claude.ai/code/session_016XhpERgAeaSiATUKTdFgci
</commit_message>
<xml_diff>
--- a/Naked_Denver_Contact_Directory_Combined.xlsx
+++ b/Naked_Denver_Contact_Directory_Combined.xlsx
@@ -25024,7 +25024,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F120"/>
+  <dimension ref="A1:F128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -25422,3456 +25422,3712 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Evergreen Dev Co</t>
+          <t>Koelbel and Company</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>4965 Washington St (Globeville)</t>
+          <t>Rendezvous Colorado (continued phases)</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>4965 Washington St, Denver (Globeville)</t>
+          <t>Winter Park, CO</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Affordable Mixed-Use – 170 units, 5-story, $132M + library</t>
+          <t>Townhomes / Single-Family / Mixed-Use Master Plan</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Under Construction (groundbreaking Jan 2026); completion fall 2027</t>
+          <t>Ongoing; Idlewild Park opened 2025</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>https://yieldpro.com/2026/01/4965-washington-street/</t>
+          <t>https://www.rendezvouscolorado.com/about-koelbel/</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Evergreen Dev Co</t>
+          <t>McWhinney</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>The Ford Apartments</t>
+          <t>Mountain Brook Flats</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Baker neighborhood, Denver</t>
+          <t>Longmont, CO</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Affordable Multifamily – 60 units, 6-story</t>
+          <t>Luxury Multifamily – 200 units, $71M</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Groundbreaking anticipated early 2026</t>
+          <t>Construction began December 2025; delivery 2027</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>https://www.evergreenreg.com/blog/evergreen-real-estate-group-announces-new-affordable-housing-community-near-denver-health-hospital-campus/</t>
+          <t>http://livmarkcommunities.com/2025/12/livmark-communities-and-mcwhinney-announce-groundbreaking-of-mountain-brook-flats-in-longmont/</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Evergreen Dev Co</t>
+          <t>McWhinney</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Superblock Industrial</t>
+          <t>Avenue South (Centerra)</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Denver Airport submarket</t>
+          <t>Loveland, CO</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Industrial – 279,374 SF, 2 buildings</t>
+          <t>Mixed-Use Master Plan – 360,000 SF + 1,750 residential units</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Groundbreaking 2025; completion Q1 2026</t>
+          <t>Groundbreaking Nov 2025; residential 2027</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>https://milehighcre.com/evergreen-devco-breaks-ground-on-final-industrial-site-in-airport-submarket/</t>
+          <t>https://www.commercialsearch.com/news/prism-places-mcwhinney-plan-mixed-use-districts-near-denver/</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Koelbel and Company</t>
+          <t>MGL Partners</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Rendezvous Colorado (continued phases)</t>
+          <t>Iliff Apartments</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Winter Park, CO</t>
+          <t>4750 E. Iliff Ave, Denver (University Hills)</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Townhomes / Single-Family / Mixed-Use Master Plan</t>
+          <t>Affordable Senior Housing – 50 units (62+), 4-story</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Ongoing; Idlewild Park opened 2025</t>
+          <t>Under Construction; completion August 2026</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>https://www.rendezvouscolorado.com/about-koelbel/</t>
+          <t>https://milehighcre.com/mgl-partners-breaks-ground-on-iliff-apartments/</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>McWhinney</t>
+          <t>RedPeak</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Mountain Brook Flats</t>
+          <t>The Allyson Townhomes</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Longmont, CO</t>
+          <t>532 Golfers Way, Denver (Lowry)</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Luxury Multifamily – 200 units, $71M</t>
+          <t>For-Rent Townhomes – 49 units (3BR/4BR)</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Construction began December 2025; delivery 2027</t>
+          <t>Completed / Open for lease-up 2025</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>http://livmarkcommunities.com/2025/12/livmark-communities-and-mcwhinney-announce-groundbreaking-of-mountain-brook-flats-in-longmont/</t>
+          <t>https://redpeak.com/the-allyson-redpeaks-stunning-new-townhomes-in-denver-now-available-for-immediate-move-in/</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>McWhinney</t>
+          <t>The Continuum Company</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Avenue South (Centerra)</t>
+          <t>9+CO</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Loveland, CO</t>
+          <t>9th Ave &amp; Colorado Blvd, Denver</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Mixed-Use Master Plan – 360,000 SF + 1,750 residential units</t>
+          <t>Mixed-Use – 11.6 acres (retail, residential, office)</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Groundbreaking Nov 2025; residential 2027</t>
+          <t>Active – recapitalized Feb 2025 ($92.5M)</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>https://www.commercialsearch.com/news/prism-places-mcwhinney-plan-mixed-use-districts-near-denver/</t>
+          <t>https://therealdeal.com/national/denver/2025/02/05/m-carlton-shell-out-93m-for-denver-office-retail-project/</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>MGL Partners</t>
+          <t>The Nichols Partnership</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Iliff Apartments</t>
+          <t>Cherry Creek North Condo/Retail</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>4750 E. Iliff Ave, Denver (University Hills)</t>
+          <t>Cherry Creek North, Denver</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Affordable Senior Housing – 50 units (62+), 4-story</t>
+          <t>Mixed-Use – 4-story condos + ground-floor retail</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Under Construction; completion August 2026</t>
+          <t>Rezoning approved April 2026; pre-development</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>https://milehighcre.com/mgl-partners-breaks-ground-on-iliff-apartments/</t>
+          <t>https://thecherrycreeknews.com/city-council-approves-high-density-development-cherry-creek/</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>RedPeak</t>
+          <t>Trailbreak Partners</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>The Allyson Townhomes</t>
+          <t>Kaia Residences</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>532 Golfers Way, Denver (Lowry)</t>
+          <t>808 N. Lincoln St, Denver (Golden Triangle)</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>For-Rent Townhomes – 49 units (3BR/4BR)</t>
+          <t>Mixed-Use Multifamily – 295 units, 18-story, $160M</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Completed / Open for lease-up 2025</t>
+          <t>Under Construction (groundbreaking April 29, 2025)</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>https://redpeak.com/the-allyson-redpeaks-stunning-new-townhomes-in-denver-now-available-for-immediate-move-in/</t>
+          <t>https://milehighcre.com/trailbreak-partners-breaks-ground-on-295-unit-kaia-residences/</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>The Continuum Company</t>
+          <t>Trailbreak Partners</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>9+CO</t>
+          <t>Boulder Townhomes</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>9th Ave &amp; Colorado Blvd, Denver</t>
+          <t>Boulder, CO</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Mixed-Use – 11.6 acres (retail, residential, office)</t>
+          <t>For-Rent Townhomes</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Active – recapitalized Feb 2025 ($92.5M)</t>
+          <t>Under Construction; $44M construction loan closed</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>https://therealdeal.com/national/denver/2025/02/05/m-carlton-shell-out-93m-for-denver-office-retail-project/</t>
+          <t>https://milehighcre.com/trailbreak-partners-closes-44m-construction-loan-for-boulder-townhomes/</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>The Nichols Partnership</t>
+          <t>Urban Villages</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Cherry Creek North Condo/Retail</t>
+          <t>Populus Hotel – Denver</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Cherry Creek North, Denver</t>
+          <t>Downtown Denver</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Mixed-Use – 4-story condos + ground-floor retail</t>
+          <t>Carbon-Positive Hotel</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Rezoning approved April 2026; pre-development</t>
+          <t>Opened late 2024; operational 2025</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>https://thecherrycreeknews.com/city-council-approves-high-density-development-cherry-creek/</t>
+          <t>https://www.naiop-colorado.org/index.php?option=com_dailyplanetblog&amp;tag=-urban-villages</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Trailbreak Partners</t>
+          <t>Zocalo Community Development</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Kaia Residences</t>
+          <t>Liora at Sloan's Lake</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>808 N. Lincoln St, Denver (Golden Triangle)</t>
+          <t>3701 16th Ave, Denver (Sloan's Lake)</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Mixed-Use Multifamily – 295 units, 18-story, $160M</t>
+          <t>Affordable Multifamily – 158 units (30/50/60% AMI), $60M</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Under Construction (groundbreaking April 29, 2025)</t>
+          <t>Under Construction (fall 2025); completion ~26 months</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>https://milehighcre.com/trailbreak-partners-breaks-ground-on-295-unit-kaia-residences/</t>
+          <t>https://milehighcre.com/zocalo-to-develop-158-affordable-apartments-in-sloans-lake/</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Trailbreak Partners</t>
+          <t>LCP Development</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Boulder Townhomes</t>
+          <t>777 Grant St Office Renovation</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Boulder, CO</t>
+          <t>777 Grant St, Denver</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>For-Rent Townhomes</t>
+          <t>Office Renovation (6-story)</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Under Construction; $44M construction loan closed</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>https://milehighcre.com/trailbreak-partners-closes-44m-construction-loan-for-boulder-townhomes/</t>
+          <t>https://crej.com/news/lcp-to-renovate-denver-housing-building-into-modern-offices/</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Urban Villages</t>
+          <t>Kairoi Residential</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Populus Hotel – Denver</t>
+          <t>Kairoi Metro Center</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Downtown Denver</t>
+          <t>E. Centrepoint Dr &amp; S. Sable Blvd, Aurora</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Carbon-Positive Hotel</t>
+          <t>Luxury Multifamily (TOD) – 419 units, 5 buildings</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Opened late 2024; operational 2025</t>
+          <t>Under Construction; completion early 2026</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>https://www.naiop-colorado.org/index.php?option=com_dailyplanetblog&amp;tag=-urban-villages</t>
+          <t>https://rebusinessonline.com/kairoi-residential-obtains-joint-venture-equity-debt-financing-for-419-unit-multifamily-project-in-aurora-colorado/</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Zocalo Community Development</t>
+          <t>Kairoi Residential</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Liora at Sloan's Lake</t>
+          <t>2777 Zuni St Hotel-to-Resi Conversion</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>3701 16th Ave, Denver (Sloan's Lake)</t>
+          <t>2777 Zuni St, Denver (LoHi)</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Affordable Multifamily – 158 units (30/50/60% AMI), $60M</t>
+          <t>Residential Conversion – 434 units (former Residence Inn)</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Under Construction (fall 2025); completion ~26 months</t>
+          <t>In permitting/review as of Dec 2025</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>https://milehighcre.com/zocalo-to-develop-158-affordable-apartments-in-sloans-lake/</t>
+          <t>https://therealdeal.com/national/denver/2025/12/10/kairoi-plots-hotel-to-resi-project-in-denver/</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>LCP Development</t>
+          <t>Kairoi Residential</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>777 Grant St Office Renovation</t>
+          <t>Belmar Park Apartments</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>777 Grant St, Denver</t>
+          <t>777 S. Yarrow St, Lakewood</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Office Renovation (6-story)</t>
+          <t>Multifamily – 411 units, 6-story</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Site plan approved May 2025; pre-construction</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>https://crej.com/news/lcp-to-renovate-denver-housing-building-into-modern-offices/</t>
+          <t>https://denvergazette.com/news/lakewood-belmar-park-apartment/article_79ecc184-1b01-427a-8f8d-9d66afd38077.html</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Kairoi Residential</t>
+          <t>Mainspring</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Kairoi Metro Center</t>
+          <t>The Sudler Renovation</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>E. Centrepoint Dr &amp; S. Sable Blvd, Aurora</t>
+          <t>1576 N. Sherman St, Denver (Uptown)</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Luxury Multifamily (TOD) – 419 units, 5 buildings</t>
+          <t>Historic Office Renovation – 28,000 SF</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Under Construction; completion early 2026</t>
+          <t>Completed; 2025 Mayor's Design Award (Preservation)</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>https://rebusinessonline.com/kairoi-residential-obtains-joint-venture-equity-debt-financing-for-419-unit-multifamily-project-in-aurora-colorado/</t>
+          <t>https://businessden.com/2024/07/15/sudler-uptown-denver-renovations-mainspring/</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Kairoi Residential</t>
+          <t>Mainspring</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>2777 Zuni St Hotel-to-Resi Conversion</t>
+          <t>2718 Walnut Redevelopment</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>2777 Zuni St, Denver (LoHi)</t>
+          <t>2718 Walnut St, Denver (RiNo)</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Residential Conversion – 434 units (former Residence Inn)</t>
+          <t>Retail/Commercial Redevelopment</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>In permitting/review as of Dec 2025</t>
+          <t>Acquired Feb 2026; redevelopment underway</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>https://therealdeal.com/national/denver/2025/12/10/kairoi-plots-hotel-to-resi-project-in-denver/</t>
+          <t>https://www.nakeddenver.com/post/mainspring-acquires-2718-walnut-plans-retail-focused-redevelopment-in-rino</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Kairoi Residential</t>
+          <t>Broe Group</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Belmar Park Apartments</t>
+          <t>250 Clayton (Phase 2)</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>777 S. Yarrow St, Lakewood</t>
+          <t>250 Clayton St, Denver (Cherry Creek North)</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Multifamily – 411 units, 6-story</t>
+          <t>Class A Office + Retail – 175,000 SF, 8-story, $225M total</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Site plan approved May 2025; pre-construction</t>
+          <t>Demolition began Q1 2026; delivery Q3 2028</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>https://denvergazette.com/news/lakewood-belmar-park-apartment/article_79ecc184-1b01-427a-8f8d-9d66afd38077.html</t>
+          <t>https://www.prnewswire.com/news-releases/the-broe-group-commences-second-phase-of-225-million-cherry-creek-north-development-302749586.html</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Mainspring</t>
+          <t>BMC Investments</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>The Sudler Renovation</t>
+          <t>Cherry Lane</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>1576 N. Sherman St, Denver (Uptown)</t>
+          <t>2500 E. 1st Ave, Denver (Cherry Creek North)</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Historic Office Renovation – 28,000 SF</t>
+          <t>Mixed-Use – 379 units + 132K SF retail + 59K SF office</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Completed; 2025 Mayor's Design Award (Preservation)</t>
+          <t>Under construction; delivery Oct 2027</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>https://businessden.com/2024/07/15/sudler-uptown-denver-renovations-mainspring/</t>
+          <t>https://milehighcre.com/bmc-to-start-construction-on-cherry-lane-development/</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Mainspring</t>
+          <t>BMC Investments</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>2718 Walnut Redevelopment</t>
+          <t>Milwaukee Place</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>2718 Walnut St, Denver (RiNo)</t>
+          <t>242 Milwaukee St, Denver (Cherry Creek)</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Retail/Commercial Redevelopment</t>
+          <t>Office – 84K SF + 10K SF retail; Crusoe AI anchor</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Acquired Feb 2026; redevelopment underway</t>
+          <t>Under construction; delivery ~2027</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>https://www.nakeddenver.com/post/mainspring-acquires-2718-walnut-plans-retail-focused-redevelopment-in-rino</t>
+          <t>https://ccdmag.com/project-updates/milwaukee-place-denver/</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>Broe Group</t>
+          <t>BMC Investments</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>250 Clayton (Phase 2)</t>
+          <t>Oasis Apartments</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>250 Clayton St, Denver (Cherry Creek North)</t>
+          <t>299 Milwaukee St, Denver (Cherry Creek North)</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>Class A Office + Retail – 175,000 SF, 8-story, $225M total</t>
+          <t>Mixed-Use – 177 luxury units + 28K SF retail</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Demolition began Q1 2026; delivery Q3 2028</t>
+          <t>Under construction; topped out Mar 2026; delivery early 2027</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/the-broe-group-commences-second-phase-of-225-million-cherry-creek-north-development-302749586.html</t>
+          <t>https://ccdmag.com/latest/bmc-construction-oasis/</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>BMC Investments</t>
+          <t>Ascentris</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Cherry Lane</t>
+          <t>Cherry Creek West</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>2500 E. 1st Ave, Denver (Cherry Creek North)</t>
+          <t>West side Cherry Creek, Denver (13-acre site)</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Mixed-Use – 379 units + 132K SF retail + 59K SF office</t>
+          <t>Mixed-Use – 1.6M SF (residential, office, retail); JV with East West Partners</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Under construction; delivery Oct 2027</t>
+          <t>Closed/acquired Q4 2024; build-out 2029–2033</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>https://milehighcre.com/bmc-to-start-construction-on-cherry-lane-development/</t>
+          <t>https://www.ascentris.com/news/ascentris-and-east-west-partners-close-on-13-acre-mixed-use-development-in-denver-co</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>BMC Investments</t>
+          <t>Infinity Properties</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Milwaukee Place</t>
+          <t>Infinity Central 18</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>242 Milwaukee St, Denver (Cherry Creek)</t>
+          <t>Central 18th Ave, LoHi, Denver</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Office – 84K SF + 10K SF retail; Crusoe AI anchor</t>
+          <t>Multifamily – 121 units, 9-story + 675 SF retail</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Under construction; delivery ~2027</t>
+          <t>In final permitting (Mar 2026); construction start Nov 2026</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>https://ccdmag.com/project-updates/milwaukee-place-denver/</t>
+          <t>https://nationaltoday.com/us/co/denver/news/2026/03/11/infinity-central-18-nears-final-permits-for-121-unit-apartment-project-in-denvers-lohi/</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>BMC Investments</t>
+          <t>Century Living</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Oasis Apartments</t>
+          <t>The Stevie</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>299 Milwaukee St, Denver (Cherry Creek North)</t>
+          <t>33rd Ave &amp; Mariposa St, LoHi, Denver</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Mixed-Use – 177 luxury units + 28K SF retail</t>
+          <t>Multifamily luxury – 116 units, 5-story</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Under construction; topped out Mar 2026; delivery early 2027</t>
+          <t>Broke ground Mar 2026; delivery 2028</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>https://ccdmag.com/latest/bmc-construction-oasis/</t>
+          <t>https://www.prnewswire.com/news-releases/century-living-acquires-site-for-luxury-apartments-in-denvers-lohi-neighborhood-302708619.html</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>Ascentris</t>
+          <t>Stockdale Capital Partners</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Cherry Creek West</t>
+          <t>Avenues at Northfield</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>West side Cherry Creek, Denver (13-acre site)</t>
+          <t>8315 Northfield Blvd, Denver</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Mixed-Use – 1.6M SF (residential, office, retail); JV with East West Partners</t>
+          <t>Retail lifestyle center renovation (1.1M SF) + 1,500 multifamily units entitled</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Closed/acquired Q4 2024; build-out 2029–2033</t>
+          <t>Under renovation; completion ahead of holiday 2026</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>https://www.ascentris.com/news/ascentris-and-east-west-partners-close-on-13-acre-mixed-use-development-in-denver-co</t>
+          <t>https://stockdalecapital.com/stockdale-capital-partners-begins-extensive-transformation-of-the-shops-at-northfield/</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Infinity Properties</t>
+          <t>Mercy Housing Mountain Plains</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Infinity Central 18</t>
+          <t>901 Navajo (Native American Affordable Housing)</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Central 18th Ave, LoHi, Denver</t>
+          <t>901 Navajo St, La Alma-Lincoln Park, Denver</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Multifamily – 121 units, 9-story + 675 SF retail</t>
+          <t>Affordable Multifamily – 190 units, 7-story + healthcare clinic</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>In final permitting (Mar 2026); construction start Nov 2026</t>
+          <t>Under construction; topped out end of 2025; move-ins Jan 2027</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>https://nationaltoday.com/us/co/denver/news/2026/03/11/infinity-central-18-nears-final-permits-for-121-unit-apartment-project-in-denvers-lohi/</t>
+          <t>https://milehighcre.com/construction-begins-on-affordable-housing-project-901-navajo/</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>Century Living</t>
+          <t>Mercy Housing Mountain Plains</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>The Stevie</t>
+          <t>Astraea at Loretto Heights</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>33rd Ave &amp; Mariposa St, LoHi, Denver</t>
+          <t>2980 Pancratia St, SW Denver</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>Multifamily luxury – 116 units, 5-story</t>
+          <t>Affordable Multifamily – 100 units (families)</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Broke ground Mar 2026; delivery 2028</t>
+          <t>Broke ground 2025; opening Mar 2027</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/century-living-acquires-site-for-luxury-apartments-in-denvers-lohi-neighborhood-302708619.html</t>
+          <t>https://www.mercyhousing.org/mountain-plains/astraea/</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Stockdale Capital Partners</t>
+          <t>Urban Land Conservancy</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Avenues at Northfield</t>
+          <t>The Irving at Mile High Vista</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>8315 Northfield Blvd, Denver</t>
+          <t>3270 W. Colfax Ave, West Colfax, Denver</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Retail lifestyle center renovation (1.1M SF) + 1,500 multifamily units entitled</t>
+          <t>Affordable Multifamily – 102 units, all-electric (community land trust)</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Under renovation; completion ahead of holiday 2026</t>
+          <t>Completed / Opened Jan 22, 2026</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>https://stockdalecapital.com/stockdale-capital-partners-begins-extensive-transformation-of-the-shops-at-northfield/</t>
+          <t>https://urbanlandc.org/urban-land-conservancy-mile-high-vista-development/</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Mercy Housing Mountain Plains</t>
+          <t>Urban Land Conservancy</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>901 Navajo (Native American Affordable Housing)</t>
+          <t>South Platte Crossing</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>901 Navajo St, La Alma-Lincoln Park, Denver</t>
+          <t>Commerce City, CO</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Affordable Multifamily – 190 units, 7-story + healthcare clinic</t>
+          <t>Affordable Multifamily – 60 units, transit-oriented</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Under construction; topped out end of 2025; move-ins Jan 2027</t>
+          <t>Completed / Grand opening Jun 2025</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>https://milehighcre.com/construction-begins-on-affordable-housing-project-901-navajo/</t>
+          <t>https://urbanlandc.org/grand-opening-south-platte-crossing-commerce-city/</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Mercy Housing Mountain Plains</t>
+          <t>Bear Peak Development</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Astraea at Loretto Heights</t>
+          <t>Pinery Village Phase II</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>2980 Pancratia St, SW Denver</t>
+          <t>North Pinery Pkwy, Douglas County</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Affordable Multifamily – 100 units (families)</t>
+          <t>Mixed commercial – 53 acres (retail, medical office, industrial, flex, self-storage)</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Broke ground 2025; opening Mar 2027</t>
+          <t>Site acquired Feb 2026 for $11M; entitlements in place</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>https://www.mercyhousing.org/mountain-plains/astraea/</t>
+          <t>https://ccdmag.com/aec-industry-news/bear-peak-douglas-county/</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>Urban Land Conservancy</t>
+          <t>CP Group</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>The Irving at Mile High Vista</t>
+          <t>Denver Place</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>3270 W. Colfax Ave, West Colfax, Denver</t>
+          <t>999 18th St, Downtown Denver</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>Affordable Multifamily – 102 units, all-electric (community land trust)</t>
+          <t>Office – 930K SF, two towers (34-story &amp; 23-story)</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Completed / Opened Jan 22, 2026</t>
+          <t>Acquired Feb 2026 for $47.5M; value-add/repositioning</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>https://urbanlandc.org/urban-land-conservancy-mile-high-vista-development/</t>
+          <t>https://therealdeal.com/national/denver/2026/02/02/cp-group-picks-up-denver-place-for-nearly-48-million/</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Urban Land Conservancy</t>
+          <t>McStain Neighborhoods</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>South Platte Crossing</t>
+          <t>Arras Park</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Commerce City, CO</t>
+          <t>Thornton, CO</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Affordable Multifamily – 60 units, transit-oriented</t>
+          <t>Townhomes (from $400s)</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Completed / Grand opening Jun 2025</t>
+          <t>Active sales / under construction 2025–2026</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>https://urbanlandc.org/grand-opening-south-platte-crossing-commerce-city/</t>
+          <t>https://mcstain.com/our-neighborhoods</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>Bear Peak Development</t>
+          <t>McStain Neighborhoods</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>Pinery Village Phase II</t>
+          <t>Painted Prairie</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>North Pinery Pkwy, Douglas County</t>
+          <t>Aurora, CO (near DIA)</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Mixed commercial – 53 acres (retail, medical office, industrial, flex, self-storage)</t>
+          <t>Single-family homes, master-planned</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Site acquired Feb 2026 for $11M; entitlements in place</t>
+          <t>Active sales / under construction 2025–2026</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>https://ccdmag.com/aec-industry-news/bear-peak-douglas-county/</t>
+          <t>https://mcstain.com/our-neighborhoods</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>CP Group</t>
+          <t>McStain Neighborhoods</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Denver Place</t>
+          <t>Westerly</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>999 18th St, Downtown Denver</t>
+          <t>Erie, CO</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Office – 930K SF, two towers (34-story &amp; 23-story)</t>
+          <t>Single-family / master-planned community</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Acquired Feb 2026 for $47.5M; value-add/repositioning</t>
+          <t>Active sales / under construction 2025–2026</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>https://therealdeal.com/national/denver/2026/02/02/cp-group-picks-up-denver-place-for-nearly-48-million/</t>
+          <t>https://mcstain.com/our-neighborhoods</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>McStain Neighborhoods</t>
+          <t>Kentro Group</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Arras Park</t>
+          <t>Platt Park Mixed-Use</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Thornton, CO</t>
+          <t>NW corner of Louisiana Ave &amp; Pearl St, Denver</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Townhomes (from $400s)</t>
+          <t>Mixed-Use – 170 units + 14K SF retail + 6K SF office</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Active sales / under construction 2025–2026</t>
+          <t>Plans submitted; groundbreaking targeted 2026</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>https://mcstain.com/our-neighborhoods</t>
+          <t>https://ccdmag.com/project-updates/platt-park-kentro/</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>McStain Neighborhoods</t>
+          <t>Kentro Group</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Painted Prairie</t>
+          <t>Belcaro Shopping Center Redevelopment</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Aurora, CO (near DIA)</t>
+          <t>Belcaro Shopping Center site, Denver</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Single-family homes, master-planned</t>
+          <t>Multifamily – 350 units, 4-story wrap</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Active sales / under construction 2025–2026</t>
+          <t>Concept plan submitted Dec 2025; in review</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>https://mcstain.com/our-neighborhoods</t>
+          <t>https://ccdmag.com/project-updates/belcaro-kentro-denver/</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>McStain Neighborhoods</t>
+          <t>CoreSite</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>Westerly</t>
+          <t>DE3 Data Center</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Erie, CO</t>
+          <t>4900 Race St, Denver</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>Single-family / master-planned community</t>
+          <t>Data Center – 180K SF / 18 MW (Phase 1 of 590K SF)</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>Active sales / under construction 2025–2026</t>
+          <t>Under construction; topped out Oct 2025; available 2026</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>https://mcstain.com/our-neighborhoods</t>
+          <t>https://www.coresite.com/news/coresite-achieves-key-construction-milestone-for-new-de3-data-center-in-denver</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Kentro Group</t>
+          <t>AC Development</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Platt Park Mixed-Use</t>
+          <t>Clayworks – Building B3</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>NW corner of Louisiana Ave &amp; Pearl St, Denver</t>
+          <t>9th St &amp; Washington Ave, Downtown Golden</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Mixed-Use – 170 units + 14K SF retail + 6K SF office</t>
+          <t>Mixed-Use – 182K SF Class AA office + 10K SF restaurant</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Plans submitted; groundbreaking targeted 2026</t>
+          <t>Under construction; topped out May 2025; completion summer 2026</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>https://ccdmag.com/project-updates/platt-park-kentro/</t>
+          <t>https://milehighcre.com/clayworks-project-in-downtown-golden-tops-out/</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>Kentro Group</t>
+          <t>Sterling Ranch Development Company</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Belcaro Shopping Center Redevelopment</t>
+          <t>Parkvale (Village 4 expansion)</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Belcaro Shopping Center site, Denver</t>
+          <t>Sterling Ranch, Douglas County</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Multifamily – 350 units, 4-story wrap</t>
+          <t>Master-planned residential (part of 4,000-acre / 16,000-unit community)</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>Concept plan submitted Dec 2025; in review</t>
+          <t>Under development; #1 selling MPC in Colorado mid-2025</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>https://ccdmag.com/project-updates/belcaro-kentro-denver/</t>
+          <t>https://sterlingranchcolorado.com/happenings/blog/sterling-ranch-continues-as-colorados-top-selling-master-planned-community-2025/</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>CoreSite</t>
+          <t>Sterling Ranch Development Company</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>DE3 Data Center</t>
+          <t>Zebulon Regional Sports Complex</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>4900 Race St, Denver</t>
+          <t>Sterling Ranch area, Douglas County</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Data Center – 180K SF / 18 MW (Phase 1 of 590K SF)</t>
+          <t>Sports complex (multi-sport) + 400 acres open space</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Under construction; topped out Oct 2025; available 2026</t>
+          <t>Development underway; $1.3B projected economic impact 2026–2036</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>https://www.coresite.com/news/coresite-achieves-key-construction-milestone-for-new-de3-data-center-in-denver</t>
+          <t>https://www.douglas.co.us/douglas-county-sterling-ranch-partner-with-private-industry-for-new-regional-sports-complex/</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>AC Development</t>
+          <t>Trammell Crow Company</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>Clayworks – Building B3</t>
+          <t>Alexan Peña Station</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>9th St &amp; Washington Ave, Downtown Golden</t>
+          <t>SW corner of 64th Ave &amp; Dunkirk St, Denver</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>Mixed-Use – 182K SF Class AA office + 10K SF restaurant</t>
+          <t>Multifamily – 578 units, 2 phases, 12 buildings, 20-acre site</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>Under construction; topped out May 2025; completion summer 2026</t>
+          <t>Under construction; welcoming residents fall 2025</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>https://milehighcre.com/clayworks-project-in-downtown-golden-tops-out/</t>
+          <t>https://www.multifamilybiz.com/pressreleases/17009/berkadia_secures_8123_million_in_joint_venture_equ...</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Sterling Ranch Development Company</t>
+          <t>KDC</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Parkvale (Village 4 expansion)</t>
+          <t>Peña Station NEXT</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Sterling Ranch, Douglas County</t>
+          <t>First transit stop from DEN Airport, Denver</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Master-planned residential (part of 4,000-acre / 16,000-unit community)</t>
+          <t>Mixed-Use – 220 acres; 3M SF office, corporate campus, hospitality, retail</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Under development; #1 selling MPC in Colorado mid-2025</t>
+          <t>Active multi-phase development</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>https://sterlingranchcolorado.com/happenings/blog/sterling-ranch-continues-as-colorados-top-selling-master-planned-community-2025/</t>
+          <t>https://kdc.com/our-work/pe%C3%B1a-station-next</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>Sterling Ranch Development Company</t>
+          <t>KDC</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>Zebulon Regional Sports Complex</t>
+          <t>Santa Fe Yards at Broadway Station</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Sterling Ranch area, Douglas County</t>
+          <t>Adjacent to Broadway Station light rail, Denver</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>Sports complex (multi-sport) + 400 acres open space</t>
+          <t>Office – 1M SF build-to-suit (4 buildings) + 5.3-acre park</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>Development underway; $1.3B projected economic impact 2026–2036</t>
+          <t>Planning/marketing phase</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>https://www.douglas.co.us/douglas-county-sterling-ranch-partner-with-private-industry-for-new-regional-sports-complex/</t>
+          <t>https://kdc.com/our-work/santa-fe-yards-at-broadway-station</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Trammell Crow Company</t>
+          <t>Milender White</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Alexan Peña Station</t>
+          <t>Denver Sidewalk Enterprise Program</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>SW corner of 64th Ave &amp; Dunkirk St, Denver</t>
+          <t>Multiple neighborhoods, Denver</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Multifamily – 578 units, 2 phases, 12 buildings, 20-acre site</t>
+          <t>Public Infrastructure / Sidewalks (~$25M contract)</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Under construction; welcoming residents fall 2025</t>
+          <t>Awarded; spot repairs 2025, new sidewalk construction Dec 2025</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>https://www.multifamilybiz.com/pressreleases/17009/berkadia_secures_8123_million_in_joint_venture_equ...</t>
+          <t>https://businessden.com/2025/07/16/milender-white-sema-construction-sidewalk-contracts/</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>KDC</t>
+          <t>Alliance Construction Solutions</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>Peña Station NEXT</t>
+          <t>38th and Tennyson Apartments</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>First transit stop from DEN Airport, Denver</t>
+          <t>W. 38th Ave &amp; Tennyson St, Denver</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>Mixed-Use – 220 acres; 3M SF office, corporate campus, hospitality, retail</t>
+          <t>Mixed-Use / Multifamily – 40 units + retail</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>Active multi-phase development</t>
+          <t>Broke ground March 2024; targeted completion early 2025</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>https://kdc.com/our-work/pe%C3%B1a-station-next</t>
+          <t>https://milehighcre.com/alliance-construction-solutions-breaks-ground-at-38th-and-tennyson-in-denver/</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>KDC</t>
+          <t>Balfour Beatty</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Santa Fe Yards at Broadway Station</t>
+          <t>Arapahoe Village Military Housing – Phase 2</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Adjacent to Broadway Station light rail, Denver</t>
+          <t>Fort Carson, Colorado Springs</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Office – 1M SF build-to-suit (4 buildings) + 5.3-acre park</t>
+          <t>Military Family Housing – $67M, 56 new homes</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Planning/marketing phase</t>
+          <t>First new homes celebrated May 2025; 24 additional planned 2026</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>https://kdc.com/our-work/santa-fe-yards-at-broadway-station</t>
+          <t>https://www.businesswire.com/news/home/20250523136880/en/Balfour-Beatty-Communities-and-U.S.-Army-Fort-Carson-Celebrate-First-New-Homes-in-$67-Million-Housing-Investment</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>Milender White</t>
+          <t>Brinkman Construction</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>Denver Sidewalk Enterprise Program</t>
+          <t>Oaks Ridge at 64th</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>Multiple neighborhoods, Denver</t>
+          <t>Near 64th Ave, Denver</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>Public Infrastructure / Sidewalks (~$25M contract)</t>
+          <t>Multifamily – 168 units, 161,375 SF (4 buildings + clubhouse)</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>Awarded; spot repairs 2025, new sidewalk construction Dec 2025</t>
+          <t>Broke ground June 2025; completion Fall 2026</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>https://businessden.com/2025/07/16/milender-white-sema-construction-sidewalk-contracts/</t>
+          <t>https://brinkmanconstruction.com/news/brinkman-construction-breaks-ground-on-oaks-ridge-at-64th/</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Alliance Construction Solutions</t>
+          <t>Brinkmann Constructors</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>38th and Tennyson Apartments</t>
+          <t>Aero 70</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>W. 38th Ave &amp; Tennyson St, Denver</t>
+          <t>Aurora, CO (169-acre site)</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Mixed-Use / Multifamily – 40 units + retail</t>
+          <t>Industrial / Speculative Warehouse – 817,500 SF, 2 buildings</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Broke ground March 2024; targeted completion early 2025</t>
+          <t>Broke ground 2024–2025; under construction</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>https://milehighcre.com/alliance-construction-solutions-breaks-ground-at-38th-and-tennyson-in-denver/</t>
+          <t>https://milehighcre.com/brinkmann-constructors-shares-new-and-completed-projects/</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>Balfour Beatty</t>
+          <t>GH Phipps Construction</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>Arapahoe Village Military Housing – Phase 2</t>
+          <t>Galen College of Nursing – HCA Healthcare</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>Fort Carson, Colorado Springs</t>
+          <t>1650 S. Potomac St, Aurora</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>Military Family Housing – $67M, 56 new homes</t>
+          <t>Higher Education / Healthcare Training – 76,500 SF</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>First new homes celebrated May 2025; 24 additional planned 2026</t>
+          <t>Topped out June 2025; targeted completion mid-2025</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>https://www.businesswire.com/news/home/20250523136880/en/Balfour-Beatty-Communities-and-U.S.-Army-Fort-Carson-Celebrate-First-New-Homes-in-$67-Million-Housing-Investment</t>
+          <t>https://ghphipps.com/galen-college-of-nursing-hca-healthcare-aurora-colorado/</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Brinkman Construction</t>
+          <t>GH Phipps Construction</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Oaks Ridge at 64th</t>
+          <t>Wellington E. Webb Municipal Office Renovation</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Near 64th Ave, Denver</t>
+          <t>201 W Colfax Ave, Denver</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Multifamily – 168 units, 161,375 SF (4 buildings + clubhouse)</t>
+          <t>Municipal Office Renovation – 11 floors, $90M phased</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Broke ground June 2025; completion Fall 2026</t>
+          <t>Active / phased renovation ongoing 2025–2026</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>https://brinkmanconstruction.com/news/brinkman-construction-breaks-ground-on-oaks-ridge-at-64th/</t>
+          <t>https://ghphipps.com/projects/</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>Brinkmann Constructors</t>
+          <t>Haselden Construction</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>Aero 70</t>
+          <t>Denver Health Sam Sandos Westside Family Health Center</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>Aurora, CO (169-acre site)</t>
+          <t>Westside, Denver</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>Industrial / Speculative Warehouse – 817,500 SF, 2 buildings</t>
+          <t>Healthcare Clinic – $20M</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>Broke ground 2024–2025; under construction</t>
+          <t>Broke ground Nov 2025; under construction</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>https://milehighcre.com/brinkmann-constructors-shares-new-and-completed-projects/</t>
+          <t>https://www.axios.com/local/denver/2025/11/05/vibrant-denver-bond-projects-groundbreaking-mike-johnston</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>GH Phipps Construction</t>
+          <t>Haselden Construction</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Galen College of Nursing – HCA Healthcare</t>
+          <t>Milwaukee Place</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>1650 S. Potomac St, Aurora</t>
+          <t>Cherry Creek North, Denver</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Higher Education / Healthcare Training – 76,500 SF</t>
+          <t>Mixed-Use Office + Retail</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Topped out June 2025; targeted completion mid-2025</t>
+          <t>Under construction; targeted completion Jan 2027</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>https://ghphipps.com/galen-college-of-nursing-hca-healthcare-aurora-colorado/</t>
+          <t>https://milehighcre.com/milwaukee-place-breaks-ground-in-cherry-creek/</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>GH Phipps Construction</t>
+          <t>Hensel Phelps</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>Wellington E. Webb Municipal Office Renovation</t>
+          <t>Colorado Convention Center Expansion</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>201 W Colfax Ave, Denver</t>
+          <t>700 14th St, Denver</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>Municipal Office Renovation – 11 floors, $90M phased</t>
+          <t>Convention Center – $212M design-build</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>Active / phased renovation ongoing 2025–2026</t>
+          <t>Construction phases ongoing</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>https://ghphipps.com/projects/</t>
+          <t>https://www.henselphelps.com/</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Haselden Construction</t>
+          <t>Hensel Phelps</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Denver Health Sam Sandos Westside Family Health Center</t>
+          <t>National Western Center Horizontal Infrastructure</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Westside, Denver</t>
+          <t>National Western Complex, Denver</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Healthcare Clinic – $20M</t>
+          <t>Civic / Campus Infrastructure</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Broke ground Nov 2025; under construction</t>
+          <t>Ongoing horizontal work</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>https://www.axios.com/local/denver/2025/11/05/vibrant-denver-bond-projects-groundbreaking-mike-johnston</t>
+          <t>https://www.henselphelps.com/project/national-western-center-horizontal-integrated-contractor/</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>Haselden Construction</t>
+          <t>Hyder Construction</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>Milwaukee Place</t>
+          <t>FirstBank Headquarters Expansion</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>Cherry Creek North, Denver</t>
+          <t>Lakewood, CO</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>Mixed-Use Office + Retail</t>
+          <t>Commercial Office – 126,000 SF + 600-stall parking garage</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>Under construction; targeted completion Jan 2027</t>
+          <t>Two phases; under construction / recent completion</t>
         </is>
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>https://milehighcre.com/milwaukee-place-breaks-ground-in-cherry-creek/</t>
+          <t>https://www.hyderinc.com/projects/</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Hensel Phelps</t>
+          <t>Hyder Construction</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Colorado Convention Center Expansion</t>
+          <t>United Airlines Flight Training Center Renovation</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>700 14th St, Denver</t>
+          <t>7500 E. 35th Ave, Denver</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Convention Center – $212M design-build</t>
+          <t>Aviation / Industrial (simulator bay renovation)</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Construction phases ongoing</t>
+          <t>Under construction / recent</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>https://www.henselphelps.com/</t>
+          <t>https://www.hyderinc.com/projects/</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>Hensel Phelps</t>
+          <t>JE Dunn Construction</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>National Western Center Horizontal Infrastructure</t>
+          <t>CSU Veterinary Hospital &amp; Education Complex</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>National Western Complex, Denver</t>
+          <t>South Campus, CSU, Fort Collins</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>Civic / Campus Infrastructure</t>
+          <t>Veterinary Hospital / Education – 213,000 SF, $230M</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>Ongoing horizontal work</t>
+          <t>Near completion Feb 2026; opening Spring 2026</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>https://www.henselphelps.com/project/national-western-center-horizontal-integrated-contractor/</t>
+          <t>https://jedunn.com/projects/colorado-state-university-veterinary-hospital/</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Hyder Construction</t>
+          <t>JE Dunn Construction</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>FirstBank Headquarters Expansion</t>
+          <t>NREL Research Facility</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Lakewood, CO</t>
+          <t>Golden, CO (South Table Mountain Campus)</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Commercial Office – 126,000 SF + 600-stall parking garage</t>
+          <t>R&amp;D / Laboratory – $224M</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Two phases; under construction / recent completion</t>
+          <t>Broke ground late 2024; under construction</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>https://www.hyderinc.com/projects/</t>
+          <t>https://www.constructiondive.com/news/je-dunn-224m-doe-department-energy-project-colorado/705188/</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>Hyder Construction</t>
+          <t>JHL Constructors</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>United Airlines Flight Training Center Renovation</t>
+          <t>Talon Ridge Middle School</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>7500 E. 35th Ave, Denver</t>
+          <t>Thornton, CO (27J School District)</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>Aviation / Industrial (simulator bay renovation)</t>
+          <t>K-12 Education – 133,000 SF</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>Under construction / recent</t>
+          <t>Under construction; targeted completion 2026</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>https://www.hyderinc.com/projects/</t>
+          <t>https://ccdmag.com/project-updates/jhl-constructors-talon-ridge/</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>JE Dunn Construction</t>
+          <t>JHL Constructors</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>CSU Veterinary Hospital &amp; Education Complex</t>
+          <t>Silverthorne Recreation Center Expansion</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>South Campus, CSU, Fort Collins</t>
+          <t>Silverthorne, CO</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Veterinary Hospital / Education – 213,000 SF, $230M</t>
+          <t>Recreation – 23,000 SF addition</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Near completion Feb 2026; opening Spring 2026</t>
+          <t>Under construction; targeted completion Summer 2026</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>https://jedunn.com/projects/colorado-state-university-veterinary-hospital/</t>
+          <t>https://www.jhlconstructors.com/jhl-constructors-breaks-ground-on-the-silverthorne-recreation-expansion-project/</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>JE Dunn Construction</t>
+          <t>Mortenson</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>NREL Research Facility</t>
+          <t>Denver Summit FC Women's Soccer Stadium</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>Golden, CO (South Table Mountain Campus)</t>
+          <t>Santa Fe Yards, Denver (near I-25 &amp; S. Broadway)</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>R&amp;D / Laboratory – $224M</t>
+          <t>Sports Stadium – 14,500 seats, $225M</t>
         </is>
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>Broke ground late 2024; under construction</t>
+          <t>Preconstruction 2025; full construction Spring 2026; opening 2028</t>
         </is>
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>https://www.constructiondive.com/news/je-dunn-224m-doe-department-energy-project-colorado/705188/</t>
+          <t>https://www.mortenson.com/news-insights/denver-summit-fc-stadium-announcement</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>JHL Constructors</t>
+          <t>Mortenson</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Talon Ridge Middle School</t>
+          <t>Cherry Creek West Redevelopment</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Thornton, CO (27J School District)</t>
+          <t>1st Ave &amp; University Blvd, Denver (13 acres)</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>K-12 Education – 133,000 SF</t>
+          <t>Mixed-Use – office, residential, retail, dining (JV with Saunders)</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Under construction; targeted completion 2026</t>
+          <t>Demolition began March 2026; phased construction 2026–2029</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>https://ccdmag.com/project-updates/jhl-constructors-talon-ridge/</t>
+          <t>https://www.saundersinc.com/about/news/mortenson-saunders-named-to-lead-construction-of-cherry-creek-west-redevelopment/</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>JHL Constructors</t>
+          <t>PCL Construction</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>Silverthorne Recreation Center Expansion</t>
+          <t>AI-Ready Data Center</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>Silverthorne, CO</t>
+          <t>Southeast Denver metro (17-acre site)</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>Recreation – 23,000 SF addition</t>
+          <t>Data Center – 22.5 MW, $192M</t>
         </is>
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>Under construction; targeted completion Summer 2026</t>
+          <t>Topped out; targeted completion Summer 2027</t>
         </is>
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>https://www.jhlconstructors.com/jhl-constructors-breaks-ground-on-the-silverthorne-recreation-expansion-project/</t>
+          <t>https://www.pcl.com/us/en/newsroom/press-releases/pcl-tops-out-192-million-ai-ready-data-center-as-denvers-digital-infrastructure-demand-accelerates</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Mortenson</t>
+          <t>PCL Construction</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Denver Summit FC Women's Soccer Stadium</t>
+          <t>Summit House – MSU Denver Student Housing</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Santa Fe Yards, Denver (near I-25 &amp; S. Broadway)</t>
+          <t>12th St &amp; Auraria Pkwy, Denver</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Sports Stadium – 14,500 seats, $225M</t>
+          <t>Student Housing – 550+ beds, 12-story mass timber, $117M</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Preconstruction 2025; full construction Spring 2026; opening 2028</t>
+          <t>Broke ground Sept 2025; substantial completion March 2027</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>https://www.mortenson.com/news-insights/denver-summit-fc-stadium-announcement</t>
+          <t>https://www.pcl.com/us/en/newsroom/press-releases/pcl-construction-and-columbia-ventures-break-ground-on-msu-denvers-first-student-housing</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>Mortenson</t>
+          <t>PCL Construction</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>Cherry Creek West Redevelopment</t>
+          <t>Westminster Blvd Drinking Water Facility</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>1st Ave &amp; University Blvd, Denver (13 acres)</t>
+          <t>9988 Westminster Blvd, Westminster</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>Mixed-Use – office, residential, retail, dining (JV with Saunders)</t>
+          <t>Water Infrastructure – $190M</t>
         </is>
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>Demolition began March 2026; phased construction 2026–2029</t>
+          <t>Broke ground Sept 2025; targeted completion 2028</t>
         </is>
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>https://www.saundersinc.com/about/news/mortenson-saunders-named-to-lead-construction-of-cherry-creek-west-redevelopment/</t>
+          <t>https://www.pcl.com/us/en/newsroom/press-releases/pcl-construction-breaks-ground-on-190-million-contract-for-state-of-the-art-drinking-water-facility</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>PCL Construction</t>
+          <t>Pinkard Construction</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>AI-Ready Data Center</t>
+          <t>akin Golden Triangle</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Southeast Denver metro (17-acre site)</t>
+          <t>Bannock St, Golden Triangle, Denver</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Data Center – 22.5 MW, $192M</t>
+          <t>Luxury Multifamily – 98 units, 12-story</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Topped out; targeted completion Summer 2027</t>
+          <t>Topped out 2024; completing finishes / targeted completion 2025</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>https://www.pcl.com/us/en/newsroom/press-releases/pcl-tops-out-192-million-ai-ready-data-center-as-denvers-digital-infrastructure-demand-accelerates</t>
+          <t>https://www.pinkardbuilds.com/pinkard-projects/akin-golden-triangle</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>PCL Construction</t>
+          <t>Pinkard Construction</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>Summit House – MSU Denver Student Housing</t>
+          <t>The Irving at Mile High Vista</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>12th St &amp; Auraria Pkwy, Denver</t>
+          <t>3270 W. Colfax Ave, Denver</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>Student Housing – 550+ beds, 12-story mass timber, $117M</t>
+          <t>Affordable Multifamily – 102 units</t>
         </is>
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>Broke ground Sept 2025; substantial completion March 2027</t>
+          <t>Completed Jan 2026</t>
         </is>
       </c>
       <c r="F79" s="3" t="inlineStr">
         <is>
-          <t>https://www.pcl.com/us/en/newsroom/press-releases/pcl-construction-and-columbia-ventures-break-ground-on-msu-denvers-first-student-housing</t>
+          <t>https://www.jeffcobdb.com/2026/01/30/pinkard-completes-affordable-housing-project-in-denver/</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>PCL Construction</t>
+          <t>Saunders Construction</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Westminster Blvd Drinking Water Facility</t>
+          <t>Cherry Creek West Redevelopment</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>9988 Westminster Blvd, Westminster</t>
+          <t>1st Ave &amp; University Blvd, Denver (13 acres)</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Water Infrastructure – $190M</t>
+          <t>Mixed-Use – office, housing, retail, dining (JV with Mortenson)</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Broke ground Sept 2025; targeted completion 2028</t>
+          <t>Demolition began March 2026; phased construction 2026–2029</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>https://www.pcl.com/us/en/newsroom/press-releases/pcl-construction-breaks-ground-on-190-million-contract-for-state-of-the-art-drinking-water-facility</t>
+          <t>https://www.saundersinc.com/about/news/mortenson-saunders-named-to-lead-construction-of-cherry-creek-west-redevelopment/</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>Pinkard Construction</t>
+          <t>Turner Construction</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>akin Golden Triangle</t>
+          <t>Denver Broncos Training HQ</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>Bannock St, Golden Triangle, Denver</t>
+          <t>Englewood, CO (26-acre site)</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>Luxury Multifamily – 98 units, 12-story</t>
+          <t>Sports / Training Facility – 320,000+ SF</t>
         </is>
       </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
-          <t>Topped out 2024; completing finishes / targeted completion 2025</t>
+          <t>Under construction; targeted completion ahead of 2026 NFL season</t>
         </is>
       </c>
       <c r="F81" s="3" t="inlineStr">
         <is>
-          <t>https://www.pinkardbuilds.com/pinkard-projects/akin-golden-triangle</t>
+          <t>https://www.constructiondive.com/news/denver-broncos-turner-training-headquarters/725752/</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Pinkard Construction</t>
+          <t>Turner Construction</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>The Irving at Mile High Vista</t>
+          <t>Agilent Technologies Pharmaceutical Manufacturing Plant</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>3270 W. Colfax Ave, Denver</t>
+          <t>Frederick, CO (near Boulder)</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>Affordable Multifamily – 102 units</t>
+          <t>Pharmaceutical Manufacturing – 200,000 SF, $725M</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Completed Jan 2026</t>
+          <t>Under construction; targeted completion 2026</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>https://www.jeffcobdb.com/2026/01/30/pinkard-completes-affordable-housing-project-in-denver/</t>
+          <t>https://www.turnerconstruction.com/insights/agilent-technologies-selects-turner-to-build-725-million-pharmaceutical-manufacturing-plant-in-fred</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>Saunders Construction</t>
+          <t>Davis Partnership Architects</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>Cherry Creek West Redevelopment</t>
+          <t>3850 Blake Street Multifamily</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>1st Ave &amp; University Blvd, Denver (13 acres)</t>
+          <t>3850 Blake St, Denver (RiNo)</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>Mixed-Use – office, housing, retail, dining (JV with Mortenson)</t>
+          <t>Multifamily – 310 units</t>
         </is>
       </c>
       <c r="E83" s="3" t="inlineStr">
         <is>
-          <t>Demolition began March 2026; phased construction 2026–2029</t>
+          <t>Under Construction (broke ground 2025)</t>
         </is>
       </c>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>https://www.saundersinc.com/about/news/mortenson-saunders-named-to-lead-construction-of-cherry-creek-west-redevelopment/</t>
+          <t>https://ccdmag.com/project-updates/formativ-3850-denver/</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Turner Construction</t>
+          <t>KTGY</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>Denver Broncos Training HQ</t>
+          <t>Aura Arts District</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>Englewood, CO (26-acre site)</t>
+          <t>505 N. Lipan St, Denver</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>Sports / Training Facility – 320,000+ SF</t>
+          <t>Multifamily – 333 units, 6-story podium</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Under construction; targeted completion ahead of 2026 NFL season</t>
+          <t>Completed 2025</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>https://www.constructiondive.com/news/denver-broncos-turner-training-headquarters/725752/</t>
+          <t>https://ktgy.com/ktgy-shapes-the-future-of-high-density-living-in-denver-metro/</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>Turner Construction</t>
+          <t>KTGY</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>Agilent Technologies Pharmaceutical Manufacturing Plant</t>
+          <t>Fellow at Fitz</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>Frederick, CO (near Boulder)</t>
+          <t>12600 E. Colfax Ave, Aurora</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>Pharmaceutical Manufacturing – 200,000 SF, $725M</t>
+          <t>Multifamily – 413 units, 7-story</t>
         </is>
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>Under construction; targeted completion 2026</t>
+          <t>Completed 2025</t>
         </is>
       </c>
       <c r="F85" s="3" t="inlineStr">
         <is>
-          <t>https://www.turnerconstruction.com/insights/agilent-technologies-selects-turner-to-build-725-million-pharmaceutical-manufacturing-plant-in-fred</t>
+          <t>https://ktgy.com/Work/fellow-at-fitz/</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Davis Partnership Architects</t>
+          <t>Populous</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>3850 Blake Street Multifamily</t>
+          <t>Sue Anschutz-Rodgers Livestock Center</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>3850 Blake St, Denver (RiNo)</t>
+          <t>National Western Center, Denver</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>Multifamily – 310 units</t>
+          <t>Agricultural / Civic / Event Venue</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Under Construction (broke ground 2025)</t>
+          <t>Completed; ribbon cut Dec. 5, 2025</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>https://ccdmag.com/project-updates/formativ-3850-denver/</t>
+          <t>https://populous.com/projects/sue-anschutz-rodgers-livestock-center</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>KTGY</t>
+          <t>Populous</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>Aura Arts District</t>
+          <t>Denver Summit FC NWSL Stadium</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>505 N. Lipan St, Denver</t>
+          <t>709 S. Delaware St (Santa Fe Yards), Denver</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>Multifamily – 333 units, 6-story podium</t>
+          <t>Sports Stadium – 14,500 seats</t>
         </is>
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>Completed 2025</t>
+          <t>Approved; construction begins May 2026; opening Feb. 2028</t>
         </is>
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>https://ktgy.com/ktgy-shapes-the-future-of-high-density-living-in-denver-metro/</t>
+          <t>https://ccdmag.com/latest/denver-soccer-nwsl/</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>KTGY</t>
+          <t>Gensler</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>Fellow at Fitz</t>
+          <t>Petroleum Building Conversion</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>12600 E. Colfax Ave, Aurora</t>
+          <t>110 16th St, Denver</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>Multifamily – 413 units, 7-story</t>
+          <t>Adaptive Reuse / Residential – 178 units, 14-story</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>Completed 2025</t>
+          <t>Permitting; groundbreaking Spring 2026; completion Summer 2027</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>https://ktgy.com/Work/fellow-at-fitz/</t>
+          <t>https://ccdmag.com/project-updates/petroleum-building/</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>Populous</t>
+          <t>HOK</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>Sue Anschutz-Rodgers Livestock Center</t>
+          <t>Denver Broncos Training Facility &amp; HQ</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>National Western Center, Denver</t>
+          <t>13655 Broncos Pkwy, Englewood</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>Agricultural / Civic / Event Venue</t>
+          <t>Sports / Corporate HQ – 205,000 SF, 3-story</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>Completed; ribbon cut Dec. 5, 2025</t>
+          <t>Under Construction; opening 2026</t>
         </is>
       </c>
       <c r="F89" s="3" t="inlineStr">
         <is>
-          <t>https://populous.com/projects/sue-anschutz-rodgers-livestock-center</t>
+          <t>https://www.hok.com/projects/view/denver-broncos-training-facility-and-headquarters/</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Populous</t>
+          <t>DLR Group</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>Denver Summit FC NWSL Stadium</t>
+          <t>T3 RiNo (Mass Timber Office)</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>709 S. Delaware St (Santa Fe Yards), Denver</t>
+          <t>3500 Blake St, Denver</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>Sports Stadium – 14,500 seats</t>
+          <t>Office – 239,000 SF, 6-story mass timber + retail</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>Approved; construction begins May 2026; opening Feb. 2028</t>
+          <t>Completed January 2025</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>https://ccdmag.com/latest/denver-soccer-nwsl/</t>
+          <t>https://www.dlrgroup.com/work/hines-t3-rino/</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>Gensler</t>
+          <t>DLR Group</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>Petroleum Building Conversion</t>
+          <t>Hyatt Regency Denver Renovation</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>110 16th St, Denver</t>
+          <t>650 15th St, Denver</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>Adaptive Reuse / Residential – 178 units, 14-story</t>
+          <t>Hotel Renovation – $70M</t>
         </is>
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>Permitting; groundbreaking Spring 2026; completion Summer 2027</t>
+          <t>Completed March 2026</t>
         </is>
       </c>
       <c r="F91" s="3" t="inlineStr">
         <is>
-          <t>https://ccdmag.com/project-updates/petroleum-building/</t>
+          <t>https://hoteldesigns.net/industry-news/sneak-peek-the-transformation-of-hyatt-regency-denver/</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>HOK</t>
+          <t>Cuningham</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>Denver Broncos Training Facility &amp; HQ</t>
+          <t>Central Park Urban Living Flats</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>13655 Broncos Pkwy, Englewood</t>
+          <t>Central Park Neighborhood, Denver</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Sports / Corporate HQ – 205,000 SF, 3-story</t>
+          <t>Affordable Condominiums – 132 units</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>Under Construction; opening 2026</t>
+          <t>Completed / Grand Opening July 14, 2025</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>https://www.hok.com/projects/view/denver-broncos-training-facility-and-headquarters/</t>
+          <t>https://cuningham.com/news/first-100-percent-affordable-condo-project-opens-denver</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>DLR Group</t>
+          <t>OZ Architecture</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>T3 RiNo (Mass Timber Office)</t>
+          <t>Sun Valley Phase 3 – Joli &amp; Flo</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>3500 Blake St, Denver</t>
+          <t>Sun Valley Neighborhood, Denver</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>Office – 239,000 SF, 6-story mass timber + retail</t>
+          <t>Affordable Housing + Mixed-Use (food incubator)</t>
         </is>
       </c>
       <c r="E93" s="3" t="inlineStr">
         <is>
-          <t>Completed January 2025</t>
+          <t>Under Construction (mid-construction 2025)</t>
         </is>
       </c>
       <c r="F93" s="3" t="inlineStr">
         <is>
-          <t>https://www.dlrgroup.com/work/hines-t3-rino/</t>
+          <t>https://ozarch.com/our-work</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>DLR Group</t>
+          <t>OZ Architecture</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>Hyatt Regency Denver Renovation</t>
+          <t>The Ayden</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>650 15th St, Denver</t>
+          <t>4228 Kalamath St, Denver (Sunnyside)</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Hotel Renovation – $70M</t>
+          <t>Multifamily – 117 units</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>Completed March 2026</t>
+          <t>Completed / Topped Out</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>https://hoteldesigns.net/industry-news/sneak-peek-the-transformation-of-hyatt-regency-denver/</t>
+          <t>https://ozarch.com/</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>Cuningham</t>
+          <t>Perkins&amp;Will</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>Central Park Urban Living Flats</t>
+          <t>Ball Arena Improvements / KSE Neighborhood Master Plan</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>Central Park Neighborhood, Denver</t>
+          <t>1000 Chopper Cir, Denver</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr">
         <is>
-          <t>Affordable Condominiums – 132 units</t>
+          <t>Sports/Entertainment Renovation + Mixed-Use Master Plan</t>
         </is>
       </c>
       <c r="E95" s="3" t="inlineStr">
         <is>
-          <t>Completed / Grand Opening July 14, 2025</t>
+          <t>Phase 1 construction begins 2026; multi-phase through ~2050</t>
         </is>
       </c>
       <c r="F95" s="3" t="inlineStr">
         <is>
-          <t>https://cuningham.com/news/first-100-percent-affordable-condo-project-opens-denver</t>
+          <t>https://perkinswill.com/project/ball-arena-improvements/</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>OZ Architecture</t>
+          <t>SAR+ Architects</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>Sun Valley Phase 3 – Joli &amp; Flo</t>
+          <t>2700 Wewatta – Supportive Housing</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>Sun Valley Neighborhood, Denver</t>
+          <t>2700 Wewatta St, Denver (Denargo Market)</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>Affordable Housing + Mixed-Use (food incubator)</t>
+          <t>Affordable/Supportive Housing – 56 units</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>Under Construction (mid-construction 2025)</t>
+          <t>Opened Spring 2025</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>https://ozarch.com/our-work</t>
+          <t>https://sararch.com/projects/</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t>OZ Architecture</t>
+          <t>Semple Brown Design</t>
         </is>
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>The Ayden</t>
+          <t>Bruce Randolph Avenue Residences</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>4228 Kalamath St, Denver (Sunnyside)</t>
+          <t>Bruce Randolph Ave, Denver</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr">
         <is>
-          <t>Multifamily – 117 units</t>
+          <t>Residential/Affordable Housing</t>
         </is>
       </c>
       <c r="E97" s="3" t="inlineStr">
         <is>
-          <t>Completed / Topped Out</t>
+          <t>Completed; Mayor's Design Award 2025</t>
         </is>
       </c>
       <c r="F97" s="3" t="inlineStr">
         <is>
-          <t>https://ozarch.com/</t>
+          <t>https://semplebrown.com/works/</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Perkins&amp;Will</t>
+          <t>Shopworks Architecture</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>Ball Arena Improvements / KSE Neighborhood Master Plan</t>
+          <t>1650 N. Hooker St (West Colfax Affordable Housing)</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>1000 Chopper Cir, Denver</t>
+          <t>1650 N. Hooker St, Denver</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>Sports/Entertainment Renovation + Mixed-Use Master Plan</t>
+          <t>Affordable Housing – 153 units, 6-story</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>Phase 1 construction begins 2026; multi-phase through ~2050</t>
+          <t>Proposed / Concept Plan submitted 2025</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>https://perkinswill.com/project/ball-arena-improvements/</t>
+          <t>https://www.developingmycity.com/denver/news/153-unit-affordable-housing-project-proposed-for-1650-hooker-street-in-west-colfax</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
         <is>
-          <t>SAR+ Architects</t>
+          <t>Stantec</t>
         </is>
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>2700 Wewatta – Supportive Housing</t>
+          <t>Denver International Airport Great Hall</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>2700 Wewatta St, Denver (Denargo Market)</t>
+          <t>8500 Peña Blvd, Denver</t>
         </is>
       </c>
       <c r="D99" s="3" t="inlineStr">
         <is>
-          <t>Affordable/Supportive Housing – 56 units</t>
+          <t>Airport Terminal Modernization (multi-phase, $1.3B total)</t>
         </is>
       </c>
       <c r="E99" s="3" t="inlineStr">
         <is>
-          <t>Opened Spring 2025</t>
+          <t>Under Construction; east checkpoint open Aug. 2025; full completion 2028</t>
         </is>
       </c>
       <c r="F99" s="3" t="inlineStr">
         <is>
-          <t>https://sararch.com/projects/</t>
+          <t>https://www.stantec.com/en/projects/united-states-projects/d/denver-international-airport-great-hall</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>Semple Brown Design</t>
+          <t>Tryba Architects</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>Bruce Randolph Avenue Residences</t>
+          <t>National Western Center – Livestock Center</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>Bruce Randolph Ave, Denver</t>
+          <t>4655 Humboldt St, Denver</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>Residential/Affordable Housing</t>
+          <t>Agricultural / Civic Event Venue – $250M</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>Completed; Mayor's Design Award 2025</t>
+          <t>Completed; Ribbon Cut Dec. 5, 2025</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>https://semplebrown.com/works/</t>
+          <t>https://www.trybaarchitects.com/news/</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>Shopworks Architecture</t>
+          <t>Tryba Architects</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>1650 N. Hooker St (West Colfax Affordable Housing)</t>
+          <t>Former Denver Medical Depot Adaptive Reuse</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
         <is>
-          <t>1650 N. Hooker St, Denver</t>
+          <t>E. 38th Ave &amp; Steele St, Clayton, Denver</t>
         </is>
       </c>
       <c r="D101" s="3" t="inlineStr">
         <is>
-          <t>Affordable Housing – 153 units, 6-story</t>
+          <t>Adaptive Reuse – Multi-Tenant Industrial/Flex (482,700 SF on 32 acres)</t>
         </is>
       </c>
       <c r="E101" s="3" t="inlineStr">
         <is>
-          <t>Proposed / Concept Plan submitted 2025</t>
+          <t>Under Construction (commenced Spring 2025)</t>
         </is>
       </c>
       <c r="F101" s="3" t="inlineStr">
         <is>
-          <t>https://www.developingmycity.com/denver/news/153-unit-affordable-housing-project-proposed-for-1650-hooker-street-in-west-colfax</t>
+          <t>https://www.trybaarchitects.com/news/tryba-architects-to-lead-renovation-and-adaptive-re-use-of-former-denver-medical-depot</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>Stantec</t>
+          <t>KEPHART</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>Denver International Airport Great Hall</t>
+          <t>Harker Heights</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>8500 Peña Blvd, Denver</t>
+          <t>Near Denver (15 min from city center)</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>Airport Terminal Modernization (multi-phase, $1.3B total)</t>
+          <t>Multifamily – 283 units</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>Under Construction; east checkpoint open Aug. 2025; full completion 2028</t>
+          <t>Under Construction; fire Jan. 2, 2026 — rebuild status uncertain</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>https://www.stantec.com/en/projects/united-states-projects/d/denver-international-airport-great-hall</t>
+          <t>https://kephart.com/project-update-the-harker/</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>Tryba Architects</t>
+          <t>KEPHART</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>National Western Center – Livestock Center</t>
+          <t>Alta Flatirons</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
         <is>
-          <t>4655 Humboldt St, Denver</t>
+          <t>Downtown Superior, CO</t>
         </is>
       </c>
       <c r="D103" s="3" t="inlineStr">
         <is>
-          <t>Agricultural / Civic Event Venue – $250M</t>
+          <t>Mixed-Use Multifamily</t>
         </is>
       </c>
       <c r="E103" s="3" t="inlineStr">
         <is>
-          <t>Completed; Ribbon Cut Dec. 5, 2025</t>
+          <t>Under Construction / Recent</t>
         </is>
       </c>
       <c r="F103" s="3" t="inlineStr">
         <is>
-          <t>https://www.trybaarchitects.com/news/</t>
+          <t>https://kephart.com/project-update-alta-flatirons-mixed-use-multifamily-shaping-downtown-superior/</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>Tryba Architects</t>
+          <t>Kimley-Horn</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>Former Denver Medical Depot Adaptive Reuse</t>
+          <t>South Broadway Multimodal Transportation Improvements</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>E. 38th Ave &amp; Steele St, Clayton, Denver</t>
+          <t>South Broadway, Denver</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>Adaptive Reuse – Multi-Tenant Industrial/Flex (482,700 SF on 32 acres)</t>
+          <t>Transportation / Multimodal (14 intersections, protected bike lane)</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>Under Construction (commenced Spring 2025)</t>
+          <t>Complete — 2025 ACEC Colorado Merit Award</t>
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>https://www.trybaarchitects.com/news/tryba-architects-to-lead-renovation-and-adaptive-re-use-of-former-denver-medical-depot</t>
+          <t>https://www.kimley-horn.com/project/transforming-multimodal-transportation-denvers-south-broadway/</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
         <is>
-          <t>KEPHART</t>
+          <t>Kimley-Horn</t>
         </is>
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>Harker Heights</t>
+          <t>Gateway Park Mixed-Use Business Park (on-call)</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
         <is>
-          <t>Near Denver (15 min from city center)</t>
+          <t>Denver/Aurora (I-70 &amp; Tower Rd area)</t>
         </is>
       </c>
       <c r="D105" s="3" t="inlineStr">
         <is>
-          <t>Multifamily – 283 units</t>
+          <t>Mixed-Use Development / On-Call Civil Engineering</t>
         </is>
       </c>
       <c r="E105" s="3" t="inlineStr">
         <is>
-          <t>Under Construction; fire Jan. 2, 2026 — rebuild status uncertain</t>
+          <t>Ongoing since 2003; active 2025–2026</t>
         </is>
       </c>
       <c r="F105" s="3" t="inlineStr">
         <is>
-          <t>https://kephart.com/project-update-the-harker/</t>
+          <t>https://www.kimley-horn.com/project/gateway-park-mixed-use-business-park/</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>KEPHART</t>
+          <t>Galloway &amp; Company</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>Alta Flatirons</t>
+          <t>56th &amp; Dunkirk Multifamily Apartments</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>Downtown Superior, CO</t>
+          <t>56th Ave &amp; Dunkirk St, Denver</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>Mixed-Use Multifamily</t>
+          <t>Multifamily – 207 units, 5-story, 157,500 SF modular</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
         <is>
-          <t>Under Construction / Recent</t>
+          <t>Recently completed / late 2024–2025</t>
         </is>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>https://kephart.com/project-update-alta-flatirons-mixed-use-multifamily-shaping-downtown-superior/</t>
+          <t>https://gallowayus.com/project/56th-dunkirk/</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
         <is>
-          <t>Kimley-Horn</t>
+          <t>Galloway &amp; Company</t>
         </is>
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t>South Broadway Multimodal Transportation Improvements</t>
+          <t>Broadway &amp; Yale Mixed-Use Development</t>
         </is>
       </c>
       <c r="C107" s="3" t="inlineStr">
         <is>
-          <t>South Broadway, Denver</t>
+          <t>Broadway &amp; Yale Ave, Denver</t>
         </is>
       </c>
       <c r="D107" s="3" t="inlineStr">
         <is>
-          <t>Transportation / Multimodal (14 intersections, protected bike lane)</t>
+          <t>Mixed-Use / Multifamily Residential</t>
         </is>
       </c>
       <c r="E107" s="3" t="inlineStr">
         <is>
-          <t>Complete — 2025 ACEC Colorado Merit Award</t>
+          <t>Design/development phase; active 2025</t>
         </is>
       </c>
       <c r="F107" s="3" t="inlineStr">
         <is>
-          <t>https://www.kimley-horn.com/project/transforming-multimodal-transportation-denvers-south-broadway/</t>
+          <t>https://gallowayus.com/project/broadway-yale/</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>Kimley-Horn</t>
+          <t>KL&amp;A Engineers and Builders</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>Gateway Park Mixed-Use Business Park (on-call)</t>
+          <t>Ball Arena District – Mass Timber Residential Towers</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>Denver/Aurora (I-70 &amp; Tower Rd area)</t>
+          <t>Ball Arena District, Denver</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>Mixed-Use Development / On-Call Civil Engineering</t>
+          <t>Structural Engineering / Mass Timber Residential (2 towers)</t>
         </is>
       </c>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>Ongoing since 2003; active 2025–2026</t>
+          <t>Design/pre-construction; selected for Denver Embodied Carbon Pilot 2025–2026</t>
         </is>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>https://www.kimley-horn.com/project/gateway-park-mixed-use-business-park/</t>
+          <t>https://nyrej.com/kla-designs-two-mass-timber-structures-for-new-55-acre-development-around-ball-arena</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
         <is>
-          <t>Galloway &amp; Company</t>
+          <t>KL&amp;A Engineers and Builders</t>
         </is>
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>56th &amp; Dunkirk Multifamily Apartments</t>
+          <t>Return to Form – 12-Story Mass Timber Multifamily</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
         <is>
-          <t>56th Ave &amp; Dunkirk St, Denver</t>
+          <t>Denver (Katz Development)</t>
         </is>
       </c>
       <c r="D109" s="3" t="inlineStr">
         <is>
-          <t>Multifamily – 207 units, 5-story, 157,500 SF modular</t>
+          <t>Structural Engineering / Multifamily + Retail (tallest mass timber in CO)</t>
         </is>
       </c>
       <c r="E109" s="3" t="inlineStr">
         <is>
-          <t>Recently completed / late 2024–2025</t>
+          <t>In development; USDA/Softwood Lumber Board award recipient</t>
         </is>
       </c>
       <c r="F109" s="3" t="inlineStr">
         <is>
-          <t>https://gallowayus.com/project/56th-dunkirk/</t>
+          <t>https://ccdmag.com/featured/tallest-mass-timber-structure-colorado/</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>Galloway &amp; Company</t>
+          <t>Raptor Civil Engineering</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>Broadway &amp; Yale Mixed-Use Development</t>
+          <t>Ochiltree Block Infill – The Griffin</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>Broadway &amp; Yale Ave, Denver</t>
+          <t>2935 Zuni St, Denver</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>Mixed-Use / Multifamily Residential</t>
+          <t>Civil Engineering / Adaptive Reuse + New Construction (32 new + 12 renovated units + retail)</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr">
         <is>
-          <t>Design/development phase; active 2025</t>
+          <t>Complete — 2025 Historic Denver Remix Award winner</t>
         </is>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>https://gallowayus.com/project/broadway-yale/</t>
+          <t>https://ccdmag.com/aec-industry-news/ochiltree-denver-award/</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
         <is>
-          <t>KL&amp;A Engineers and Builders</t>
+          <t>Martin/Martin Consulting Engineers</t>
         </is>
       </c>
       <c r="B111" s="3" t="inlineStr">
         <is>
-          <t>Ball Arena District – Mass Timber Residential Towers</t>
+          <t>16th Street Mall Reconstruction</t>
         </is>
       </c>
       <c r="C111" s="3" t="inlineStr">
         <is>
-          <t>Ball Arena District, Denver</t>
+          <t>16th Street Mall, Denver (12.5 blocks)</t>
         </is>
       </c>
       <c r="D111" s="3" t="inlineStr">
         <is>
-          <t>Structural Engineering / Mass Timber Residential (2 towers)</t>
+          <t>Civil Engineering / Urban Infrastructure Reconstruction</t>
         </is>
       </c>
       <c r="E111" s="3" t="inlineStr">
         <is>
-          <t>Design/pre-construction; selected for Denver Embodied Carbon Pilot 2025–2026</t>
+          <t>Substantially complete — 2026 ACEC Colorado Grand Conceptor Award winner</t>
         </is>
       </c>
       <c r="F111" s="3" t="inlineStr">
         <is>
-          <t>https://nyrej.com/kla-designs-two-mass-timber-structures-for-new-55-acre-development-around-ball-arena</t>
+          <t>https://www.martinmartin.com/projects/city-and-county-of-denver-16th-street-reconstruction/</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>KL&amp;A Engineers and Builders</t>
+          <t>Martin/Martin Consulting Engineers</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>Return to Form – 12-Story Mass Timber Multifamily</t>
+          <t>Denver International Airport Great Hall</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>Denver (Katz Development)</t>
+          <t>8500 Peña Blvd, Denver</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t>Structural Engineering / Multifamily + Retail (tallest mass timber in CO)</t>
+          <t>Structural/Civil Engineering / Airport Terminal</t>
         </is>
       </c>
       <c r="E112" s="2" t="inlineStr">
         <is>
-          <t>In development; USDA/Softwood Lumber Board award recipient</t>
+          <t>Phase 3 under construction; east side 2026, south end 2028</t>
         </is>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>https://ccdmag.com/featured/tallest-mass-timber-structure-colorado/</t>
+          <t>https://www.martinmartin.com/project/denver-international-airport-great-hall/</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="3" t="inlineStr">
         <is>
-          <t>Raptor Civil Engineering</t>
+          <t>IMEG</t>
         </is>
       </c>
       <c r="B113" s="3" t="inlineStr">
         <is>
-          <t>Ochiltree Block Infill – The Griffin</t>
+          <t>Denver Water Operations Complex Redevelopment</t>
         </is>
       </c>
       <c r="C113" s="3" t="inlineStr">
         <is>
-          <t>2935 Zuni St, Denver</t>
+          <t>Denver Water Campus, Denver</t>
         </is>
       </c>
       <c r="D113" s="3" t="inlineStr">
         <is>
-          <t>Civil Engineering / Adaptive Reuse + New Construction (32 new + 12 renovated units + retail)</t>
+          <t>MEP/Structural Engineering – 186,000 SF LEED Platinum Net-Zero Admin + 36-acre campus ($205M)</t>
         </is>
       </c>
       <c r="E113" s="3" t="inlineStr">
         <is>
-          <t>Complete — 2025 Historic Denver Remix Award winner</t>
+          <t>Complete / Award-winning</t>
         </is>
       </c>
       <c r="F113" s="3" t="inlineStr">
         <is>
-          <t>https://ccdmag.com/aec-industry-news/ochiltree-denver-award/</t>
+          <t>https://imegcorp.com/library/denver-water-operations-complex-redevelopment/</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>Martin/Martin Consulting Engineers</t>
+          <t>Craft Civil Design</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>16th Street Mall Reconstruction</t>
+          <t>Tapestry Affordable Housing</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>16th Street Mall, Denver (12.5 blocks)</t>
+          <t>1799 Pennsylvania St, Denver (Uptown)</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>Civil Engineering / Urban Infrastructure Reconstruction</t>
+          <t>Civil Engineering / Affordable Multifamily – 72 units, 5-story + childcare + health clinic</t>
         </is>
       </c>
       <c r="E114" s="2" t="inlineStr">
         <is>
-          <t>Substantially complete — 2026 ACEC Colorado Grand Conceptor Award winner</t>
+          <t>Under construction (broke ground Dec 15, 2025); est. completion late 2027</t>
         </is>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>https://www.martinmartin.com/projects/city-and-county-of-denver-16th-street-reconstruction/</t>
+          <t>https://www.bisnow.com/denver/news/deal-sheet/affordable-housing-project-with-childcare-clinic-breaks-ground-the-denver-deal-sheet-132412</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
         <is>
-          <t>Martin/Martin Consulting Engineers</t>
+          <t>ME Engineers</t>
         </is>
       </c>
       <c r="B115" s="3" t="inlineStr">
         <is>
-          <t>Denver International Airport Great Hall</t>
+          <t>201 Fillmore – Class A Office Building</t>
         </is>
       </c>
       <c r="C115" s="3" t="inlineStr">
         <is>
-          <t>8500 Peña Blvd, Denver</t>
+          <t>201 Fillmore St, Cherry Creek North, Denver</t>
         </is>
       </c>
       <c r="D115" s="3" t="inlineStr">
         <is>
-          <t>Structural/Civil Engineering / Airport Terminal</t>
+          <t>MEP Engineering / 8-story, 140,000 SF Class A Office + dining + rooftop</t>
         </is>
       </c>
       <c r="E115" s="3" t="inlineStr">
         <is>
-          <t>Phase 3 under construction; east side 2026, south end 2028</t>
+          <t>Under construction / completion targeted Q3 2025</t>
         </is>
       </c>
       <c r="F115" s="3" t="inlineStr">
         <is>
-          <t>https://www.martinmartin.com/project/denver-international-airport-great-hall/</t>
+          <t>https://schnitzerwest.com/projects/201-fillmore/</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>IMEG</t>
+          <t>RK Industries</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>Denver Water Operations Complex Redevelopment</t>
+          <t>New Aurora Headquarters Campus</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>Denver Water Campus, Denver</t>
+          <t>Aurora, CO</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>MEP/Structural Engineering – 186,000 SF LEED Platinum Net-Zero Admin + 36-acre campus ($205M)</t>
+          <t>Construction Engineering / HQ Facility – 154,488 SF</t>
         </is>
       </c>
       <c r="E116" s="2" t="inlineStr">
         <is>
-          <t>Complete / Award-winning</t>
+          <t>Announced Sept 2025; active construction; 1,786 jobs projected</t>
         </is>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>https://imegcorp.com/library/denver-water-operations-complex-redevelopment/</t>
+          <t>https://rkindustries.com/news/rk-industries-announces-major-expansion-in-aurora-colorado-bringing-1786-new-jobs/</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="3" t="inlineStr">
         <is>
-          <t>Craft Civil Design</t>
+          <t>Stantec</t>
         </is>
       </c>
       <c r="B117" s="3" t="inlineStr">
         <is>
-          <t>Tapestry Affordable Housing</t>
+          <t>Gross Reservoir Expansion / Gross Dam Raise</t>
         </is>
       </c>
       <c r="C117" s="3" t="inlineStr">
         <is>
-          <t>1799 Pennsylvania St, Denver (Uptown)</t>
+          <t>Gross Reservoir, Boulder County</t>
         </is>
       </c>
       <c r="D117" s="3" t="inlineStr">
         <is>
-          <t>Civil Engineering / Affordable Multifamily – 72 units, 5-story + childcare + health clinic</t>
+          <t>Civil/Structural Engineering / Dam Raise – $531M (largest RCC dam raise in world)</t>
         </is>
       </c>
       <c r="E117" s="3" t="inlineStr">
         <is>
-          <t>Under construction (broke ground Dec 15, 2025); est. completion late 2027</t>
+          <t>95% complete Dec 2025; construction paused pending court ruling</t>
         </is>
       </c>
       <c r="F117" s="3" t="inlineStr">
         <is>
-          <t>https://www.bisnow.com/denver/news/deal-sheet/affordable-housing-project-with-childcare-clinic-breaks-ground-the-denver-deal-sheet-132412</t>
+          <t>https://www.stantec.com/en/projects/united-states-projects/g/gross-reservoir-expansion-dam-raise</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>ME Engineers</t>
+          <t>Evergreen Dev Co</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>201 Fillmore – Class A Office Building</t>
+          <t>The Lookout at Clear Creek Crossing</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>201 Fillmore St, Cherry Creek North, Denver</t>
+          <t>SW corner of I-70 &amp; Hwy 58, Wheat Ridge</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>MEP Engineering / 8-story, 140,000 SF Class A Office + dining + rooftop</t>
+          <t>Dining &amp; Entertainment – 3-building, 4.76 acres (Prost Brewing, food hall, restaurant)</t>
         </is>
       </c>
       <c r="E118" s="2" t="inlineStr">
         <is>
-          <t>Under construction / completion targeted Q3 2025</t>
+          <t>Approved Feb 2025; under construction; completion late 2025</t>
         </is>
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>https://schnitzerwest.com/projects/201-fillmore/</t>
+          <t>https://milehighcre.com/premier-dining-destination-breaks-ground-in-wheat-ridge/</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="3" t="inlineStr">
         <is>
-          <t>RK Industries</t>
+          <t>Evergreen Dev Co</t>
         </is>
       </c>
       <c r="B119" s="3" t="inlineStr">
         <is>
-          <t>New Aurora Headquarters Campus</t>
+          <t>Clear Creek Crossing (Outlook Apts – sold)</t>
         </is>
       </c>
       <c r="C119" s="3" t="inlineStr">
         <is>
-          <t>Aurora, CO</t>
+          <t>I-70 &amp; Hwy 58, Wheat Ridge (serves Golden/Arvada)</t>
         </is>
       </c>
       <c r="D119" s="3" t="inlineStr">
         <is>
-          <t>Construction Engineering / HQ Facility – 154,488 SF</t>
+          <t>Multifamily – 310 units (sold to Seagate for $142M); 110-acre mixed-use district ongoing</t>
         </is>
       </c>
       <c r="E119" s="3" t="inlineStr">
         <is>
-          <t>Announced Sept 2025; active construction; 1,786 jobs projected</t>
+          <t>Apartments completed &amp; sold; broader district continuing buildout</t>
         </is>
       </c>
       <c r="F119" s="3" t="inlineStr">
         <is>
-          <t>https://rkindustries.com/news/rk-industries-announces-major-expansion-in-aurora-colorado-bringing-1786-new-jobs/</t>
+          <t>https://milehighcre.com/evergreen-devco-opens-apartment-leasing-for-outlook-clear-creek-in-wheat-ridge/</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>Stantec</t>
+          <t>Evergreen Dev Co</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>Gross Reservoir Expansion / Gross Dam Raise</t>
+          <t>Green Valley Ranch &amp; Peña (56th &amp; Tower)</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>Gross Reservoir, Boulder County</t>
+          <t>56th Ave &amp; Tower Rd, Denver (Green Valley Ranch)</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>Civil/Structural Engineering / Dam Raise – $531M (largest RCC dam raise in world)</t>
+          <t>Retail – Sprouts Farmers Market-anchored shopping center</t>
         </is>
       </c>
       <c r="E120" s="2" t="inlineStr">
         <is>
-          <t>95% complete Dec 2025; construction paused pending court ruling</t>
+          <t>Operational; one outparcel remaining for lease</t>
         </is>
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>https://www.stantec.com/en/projects/united-states-projects/g/gross-reservoir-expansion-dam-raise</t>
+          <t>https://evgre.com/properties/56th-tower-denver-co</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="3" t="inlineStr">
+        <is>
+          <t>Evergreen Dev Co</t>
+        </is>
+      </c>
+      <c r="B121" s="3" t="inlineStr">
+        <is>
+          <t>Superblock Industrial</t>
+        </is>
+      </c>
+      <c r="C121" s="3" t="inlineStr">
+        <is>
+          <t>4439 N. Telluride St &amp; 17688 E. 45th Ave, Denver (Green Valley Ranch/Airport)</t>
+        </is>
+      </c>
+      <c r="D121" s="3" t="inlineStr">
+        <is>
+          <t>Industrial – 279,374 SF spec (2 buildings, 16.59 acres)</t>
+        </is>
+      </c>
+      <c r="E121" s="3" t="inlineStr">
+        <is>
+          <t>Broke ground 2024; completion Q1 2026; CBRE leasing active</t>
+        </is>
+      </c>
+      <c r="F121" s="3" t="inlineStr">
+        <is>
+          <t>https://milehighcre.com/evergreen-devco-breaks-ground-on-final-industrial-site-in-airport-submarket/</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>Evergreen Dev Co</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>Green Valley Ranch Blvd Mixed-Use Site</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>17598 Green Valley Ranch Blvd, Denver (near DIA)</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t>Mixed-Use – 68.7 acres (retail, residential, industrial); rezoned I-2</t>
+        </is>
+      </c>
+      <c r="E122" s="2" t="inlineStr">
+        <is>
+          <t>Industrial component in development; retail/residential in planning</t>
+        </is>
+      </c>
+      <c r="F122" s="2" t="inlineStr">
+        <is>
+          <t>https://evgre.com/new-mixed-use-development-proposed-on-nearly-70-acres-by-dia</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="3" t="inlineStr">
+        <is>
+          <t>Evergreen Dev Co</t>
+        </is>
+      </c>
+      <c r="B123" s="3" t="inlineStr">
+        <is>
+          <t>88th &amp; Rosemary Industrial</t>
+        </is>
+      </c>
+      <c r="C123" s="3" t="inlineStr">
+        <is>
+          <t>8705 Rosemary St, Commerce City</t>
+        </is>
+      </c>
+      <c r="D123" s="3" t="inlineStr">
+        <is>
+          <t>Industrial – 54,600 SF grade-level + ~3-acre outdoor storage yard (6.9 acres)</t>
+        </is>
+      </c>
+      <c r="E123" s="3" t="inlineStr">
+        <is>
+          <t>Construction complete; in lease-up</t>
+        </is>
+      </c>
+      <c r="F123" s="3" t="inlineStr">
+        <is>
+          <t>https://milehighcre.com/evergreen-devco-breaks-ground-on-first-industrial-building-in-colorado/</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>Evergreen Dev Co</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>RiverPark</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>7755 S. Santa Fe Dr (SW corner Mineral &amp; Santa Fe), Littleton</t>
+        </is>
+      </c>
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>Mixed-Use TOD – 33 acres; multifamily + retail pads (Daily Needs District)</t>
+        </is>
+      </c>
+      <c r="E124" s="2" t="inlineStr">
+        <is>
+          <t>Site work active; infrastructure construction begins fall 2025; completion 2027</t>
+        </is>
+      </c>
+      <c r="F124" s="2" t="inlineStr">
+        <is>
+          <t>https://evgre.com/properties/mineral-santa-fe-littleton-co</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="3" t="inlineStr">
+        <is>
+          <t>Evergreen Dev Co</t>
+        </is>
+      </c>
+      <c r="B125" s="3" t="inlineStr">
+        <is>
+          <t>4965 Washington St (Globeville)</t>
+        </is>
+      </c>
+      <c r="C125" s="3" t="inlineStr">
+        <is>
+          <t>4965 Washington St, Denver (Globeville)</t>
+        </is>
+      </c>
+      <c r="D125" s="3" t="inlineStr">
+        <is>
+          <t>Affordable Mixed-Use – 170 units, 5-story, $132M + Denver Public Library branch</t>
+        </is>
+      </c>
+      <c r="E125" s="3" t="inlineStr">
+        <is>
+          <t>Under construction (groundbreaking Jan 2026); completion fall 2027</t>
+        </is>
+      </c>
+      <c r="F125" s="3" t="inlineStr">
+        <is>
+          <t>https://yieldpro.com/2026/01/4965-washington-street/</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>Evergreen Dev Co</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>The Ford Apartments</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>Baker neighborhood, Denver</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t>Affordable Multifamily – 60 units, 6-story</t>
+        </is>
+      </c>
+      <c r="E126" s="2" t="inlineStr">
+        <is>
+          <t>Groundbreaking anticipated early 2026</t>
+        </is>
+      </c>
+      <c r="F126" s="2" t="inlineStr">
+        <is>
+          <t>https://www.evergreenreg.com/blog/evergreen-real-estate-group-announces-new-affordable-housing-community-near-denver-health-hospital-campus/</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="3" t="inlineStr">
+        <is>
+          <t>Evergreen Dev Co</t>
+        </is>
+      </c>
+      <c r="B127" s="3" t="inlineStr">
+        <is>
+          <t>Erie Highlands</t>
+        </is>
+      </c>
+      <c r="C127" s="3" t="inlineStr">
+        <is>
+          <t>SW corner of County Road 5 &amp; Erie Pkwy, Erie</t>
+        </is>
+      </c>
+      <c r="D127" s="3" t="inlineStr">
+        <is>
+          <t>Retail – 12.71-acre neighborhood retail/commercial</t>
+        </is>
+      </c>
+      <c r="E127" s="3" t="inlineStr">
+        <is>
+          <t>Site acquired Jan 2025; broke ground July 1, 2025; active construction</t>
+        </is>
+      </c>
+      <c r="F127" s="3" t="inlineStr">
+        <is>
+          <t>https://milehighcre.com/evergreen-devco-breaks-ground-on-retail-development-in-erie/</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>Evergreen Dev Co</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>Silverstone Marketplace</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t>Hwy 52 &amp; Colorado Blvd, Frederick</t>
+        </is>
+      </c>
+      <c r="D128" s="2" t="inlineStr">
+        <is>
+          <t>Retail – 35-acre shopping center; King Soopers Marketplace anchor (123,000 SF)</t>
+        </is>
+      </c>
+      <c r="E128" s="2" t="inlineStr">
+        <is>
+          <t>Substantially complete; King Soopers grand-opened May 21, 2025; 3 pads remaining</t>
+        </is>
+      </c>
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t>https://milehighcre.com/evergreen-devco-brings-first-king-soopers-to-frederick/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add developingmycity.com data: 23 projects, 17 companies, 10 contacts
https://claude.ai/code/session_016XhpERgAeaSiATUKTdFgci
</commit_message>
<xml_diff>
--- a/Naked_Denver_Contact_Directory_Combined.xlsx
+++ b/Naked_Denver_Contact_Directory_Combined.xlsx
@@ -623,7 +623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I66"/>
+  <dimension ref="A1:I89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3725,6 +3725,1087 @@
       <c r="I66" t="inlineStr">
         <is>
           <t>https://www.nakeddenver.com/projects/cherry-lane</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>High Fidelity Plaza</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>621-633 17th Street, Denver</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Downtown</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/621-633-17th-street-office-to-residential-conversion-denver</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Proposed / Financing Approved</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Office-to-residential conversion. Developer: The Luzzatto Company. Architect: HLW International.</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>~March 2026</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/621-633-17th-street-office-to-residential-conversion-denver</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Denver Energy Center Conversion</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>1625 Broadway (Tower 2), Denver</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Downtown / Golden Triangle</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/625-broadway-denver-energy-center-office-to-residential-conversion</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Proposed (Concept Plan)</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Office-to-residential conversion. Developer: The Luzzatto Company.</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>February 2026</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/625-broadway-denver-energy-center-office-to-residential-conversion</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Central Park Station Affordable Housing</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>3801 Ulster Street, Denver</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Central Park</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/rtd-central-park-station-advances-150-unit-affordable-housing-project</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Proposed (Concept Approved)</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>150-unit affordable housing + childcare. Developer: Ulysses Development Group (RTD land). Architect: SAR+.</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>~March 2026</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/rtd-central-park-station-advances-150-unit-affordable-housing-project</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Barnum Park Row Homes</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>3419 W 5th Avenue, Denver</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Barnum</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/barnum-row-home-project-west-5th-avenue-denver</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Proposed (Concept Plan)</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Row home development.</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>~March 2026</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/barnum-row-home-project-west-5th-avenue-denver</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>602 W. 29th Ave Affordable Housing</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>602 West 29th Avenue, Denver</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Five Points / Near Coors Field</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/70-unit-affordable-housing-29th-fox-denver</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Proposed (Concept Plan)</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>70-unit affordable housing. Developer: Elevation Development Group / Steele Properties. Civil: Martin/Martin.</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>~April 2026</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/70-unit-affordable-housing-29th-fox-denver</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Civic Center Next 100</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Civic Center Park, Downtown Denver</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Downtown / Civic Center</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/civic-center-park-renovation-denver-next-100</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Park renovation. Developer: City of Denver Parks &amp; Recreation. Architect: Studio Gang.</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>~March 2026</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/civic-center-park-renovation-denver-next-100</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>University Building Affordable Housing</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>910 16th Street, Denver</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Downtown</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/university-building-affordable-housing-denver</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Proposed (Concept Plan Resubmitted)</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Office-to-residential affordable conversion. Developer: Mile High Development / BMC Investments.</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>~April 2026</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/university-building-affordable-housing-denver</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Northfield Duplex Community</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>8510 Northfield Boulevard, Denver</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Northfield / Stapleton</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/northfield-denver-210-unit-duplex-development</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Proposed (Concept Plan)</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>210-unit for-rent duplex community. Developer: BB Living.</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>~March 2026</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/northfield-denver-210-unit-duplex-development</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>The James</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Evans Ave &amp; S. Gilpin St, Denver</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>University</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/the-james-evans-gilpin-denver</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Mixed-use multifamily. GC: Bristlecone Construction. Architect: Semple Brown Design.</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>~2025-2026</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/the-james-evans-gilpin-denver</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>The Berg at Shoenberg Farms</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>73rd Ave &amp; Sheridan Blvd, Westminster</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Westminster</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/the-berg-shoenberg-farms-westminster-food-hall</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Proposed / Under Development</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Food hall / entertainment / retail. Developers: Matthew Lawrence &amp; John Crays. Civil: Raptor Civil.</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>~2025-2026</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/the-berg-shoenberg-farms-westminster-food-hall</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>156-Unit Gateway Affordable Housing</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Gateway / Green Valley Ranch area, Denver</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Gateway</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/denver-health-156-unit-affordable-housing-denver-gateway</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Proposed (Urban Design Review)</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>156-unit affordable housing + childcare.</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>March 26, 2026</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/denver-health-156-unit-affordable-housing-denver-gateway</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Milepost 35 / Central Park Multifamily</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>9226 E. Northfield Boulevard, Denver</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Central Park</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/429-unit-multifamily-development-central-park-denver</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Proposed (Concept Plan)</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>429-unit multifamily.</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>~2026</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/429-unit-multifamily-development-central-park-denver</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Marieta / 1717 Washington Condos</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>1717 N. Washington Street, Denver</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Uptown / North Capitol Hill</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/project-portal/1717-washington-condos-uptown</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Condos + retail. Developer: Generation Development. Architect: Bryant Flink Architecture.</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>~2025-2026</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/project-portal/1717-washington-condos-uptown</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>799 N. Logan St Housing</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>799 N. Logan Street, Denver</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Capitol Hill</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/799-logan-governors-mansion-housing-denver</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Proposed (Concept Plan)</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Affordable housing. Developer: State of Colorado / P3 Office.</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>March 17, 2026</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/799-logan-governors-mansion-housing-denver</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>55 N. Corona Townhomes</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>55 N. Corona Street, Denver</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Speer</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/55-corona-townhomes-denver</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Proposed (Concept Plan)</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Townhomes. Developer: Milwaukee Development LLC. Architect: Points West Design. Civil: Proof Civil.</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>March 16, 2026</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/55-corona-townhomes-denver</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>1330 Leyden Street Housing</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>1330 Leyden Street, Denver</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Montclair</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/16-unit-housing-1330-leyden-street-denver</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Proposed (Concept Plan)</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>16-unit multifamily.</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>March 15, 2026</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/16-unit-housing-1330-leyden-street-denver</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Denargo Market – Building 1</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Denargo St &amp; Delgany St, Denver (RiNo)</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>RiNo</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/denargo-market-16-story-site-development-plan</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Under Review / SDP Filed</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>16-story mixed-use. Developer: Golub &amp; Company / Formativ. Architect: Goettsch Partners. Landscape: Sasaki. Civil: Martin/Martin.</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>December 2025</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/denargo-market-16-story-site-development-plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Skyline Park Redesign</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Arapahoe St between 16th &amp; 17th St, Denver</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Downtown</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/closer-look-at-downtown-denvers-massive-skyline-park-transformation</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Park redesign. Developer: City &amp; County of Denver / Downtown Denver Partnership. Architect: RIOS.</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>~February 2026</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/closer-look-at-downtown-denvers-massive-skyline-park-transformation</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Park Hill Park</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Former Park Hill Golf Course, NE Denver</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Park Hill</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/park-hill-park-framework-plan-denver</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Planning / Framework Plan Released</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Parks / Public Open Space. Architect: Sasaki.</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>~2026</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/park-hill-park-framework-plan-denver</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Denver Museum of Nature &amp; Science – Gems &amp; Minerals Hall</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>2001 Colorado Blvd, Denver</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>City Park</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/denver-museum-gems-minerals-hall-renovation-30m-closure-2026</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>$30M museum renovation.</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>~April 2026</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/denver-museum-gems-minerals-hall-renovation-30m-closure-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Swansea Recreation Center Indoor Pool</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>2581 Valentia St, Denver</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Swansea</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/swansea-recreation-center-new-indoor-pool-denver</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Completed / Opened</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Public aquatic facility. Developer: City of Denver. GC: FCI Constructors. Architect: HDR.</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>May 27, 2026</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/swansea-recreation-center-new-indoor-pool-denver</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>41st &amp; Jason Townhomes</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>W. 41st Ave &amp; Jason St, Denver</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>North Denver</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/12-unit-townhome-development-41st-jason-denver</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Proposed (Concept Plan)</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>12-unit townhomes.</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>May 27, 2026</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/12-unit-townhome-development-41st-jason-denver</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Montbello Townhomes</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Dillon St &amp; Andrews Dr, Denver</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Montbello</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/64-unit-townhome-project-northeast-denver-dillon-street</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Proposed (SDP Filed)</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>64-unit townhomes.</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>~2026</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/64-unit-townhome-project-northeast-denver-dillon-street</t>
         </is>
       </c>
     </row>
@@ -3739,7 +4820,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M167"/>
+  <dimension ref="A1:M177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12735,6 +13816,516 @@
           <t>2026-05-31</t>
         </is>
       </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>High Fidelity Plaza</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>The Luzzatto Company</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Asher Luzzatto</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>President</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr"/>
+      <c r="G168" t="inlineStr"/>
+      <c r="H168" t="inlineStr"/>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/621-633-17th-street-office-to-residential-conversion-denver</t>
+        </is>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="L168" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="M168" t="inlineStr"/>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Central Park Station Affordable Housing</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Ulysses Development Group</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Connor Larr</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>Managing Partner</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr"/>
+      <c r="G169" t="inlineStr"/>
+      <c r="H169" t="inlineStr"/>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/rtd-central-park-station-advances-150-unit-affordable-housing-project</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="M169" t="inlineStr"/>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>University Building Affordable Housing</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>BMC Investments</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Matt Joblon</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>Founding Partner &amp; CEO</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr"/>
+      <c r="G170" t="inlineStr"/>
+      <c r="H170" t="inlineStr"/>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/university-building-affordable-housing-denver</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="M170" t="inlineStr"/>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>University Building Affordable Housing</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Mile High Development</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>George Thorn</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>Principal</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr"/>
+      <c r="G171" t="inlineStr"/>
+      <c r="H171" t="inlineStr"/>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/university-building-affordable-housing-denver</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="M171" t="inlineStr"/>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Marieta / 1717 Washington Condos</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Generation Development</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Chris Lonigro</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>President</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr"/>
+      <c r="G172" t="inlineStr"/>
+      <c r="H172" t="inlineStr"/>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/project-portal/1717-washington-condos-uptown</t>
+        </is>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="L172" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="M172" t="inlineStr"/>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>602 W. 29th Ave Affordable Housing</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Elevation Development Group</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Brad Farber</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr"/>
+      <c r="G173" t="inlineStr"/>
+      <c r="H173" t="inlineStr"/>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/70-unit-affordable-housing-29th-fox-denver</t>
+        </is>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="L173" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="M173" t="inlineStr"/>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>602 W. 29th Ave Affordable Housing</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Elevation Development Group</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Brent Farber</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr"/>
+      <c r="G174" t="inlineStr"/>
+      <c r="H174" t="inlineStr"/>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/70-unit-affordable-housing-29th-fox-denver</t>
+        </is>
+      </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="K174" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="L174" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="M174" t="inlineStr"/>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>602 W. 29th Ave Affordable Housing</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Elevation Development Group</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Gregg Farber</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr"/>
+      <c r="G175" t="inlineStr"/>
+      <c r="H175" t="inlineStr"/>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/70-unit-affordable-housing-29th-fox-denver</t>
+        </is>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="L175" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="M175" t="inlineStr"/>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>The Berg at Shoenberg Farms</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Matthew Lawrence</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>Developer/Co-owner</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr"/>
+      <c r="G176" t="inlineStr"/>
+      <c r="H176" t="inlineStr"/>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/the-berg-shoenberg-farms-westminster-food-hall</t>
+        </is>
+      </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="K176" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="L176" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="M176" t="inlineStr"/>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>The Berg at Shoenberg Farms</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>John Crays</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>Developer/Co-owner</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr"/>
+      <c r="G177" t="inlineStr"/>
+      <c r="H177" t="inlineStr"/>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/the-berg-shoenberg-farms-westminster-food-hall</t>
+        </is>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="M177" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12747,7 +14338,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I298"/>
+  <dimension ref="A1:I315"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24750,6 +26341,693 @@
           <t>2026-05-31</t>
         </is>
       </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>The Luzzatto Company</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr"/>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>Office-to-residential conversion specialist; active in Denver downtown conversions</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/621-633-17th-street-office-to-residential-conversion-denver</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I299" t="inlineStr"/>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>Ulysses Development Group</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr"/>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>Denver, CO</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>Affordable housing developer; Central Park Station TOD project</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/rtd-central-park-station-advances-150-unit-affordable-housing-project</t>
+        </is>
+      </c>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I300" t="inlineStr"/>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>Elevation Development Group</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr"/>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>Denver, CO</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>Affordable housing developer; 602 W. 29th Ave project</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/70-unit-affordable-housing-29th-fox-denver</t>
+        </is>
+      </c>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I301" t="inlineStr"/>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>Mile High Development</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr"/>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>Denver, CO</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>Affordable housing / adaptive reuse developer; University Building conversion</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/university-building-affordable-housing-denver</t>
+        </is>
+      </c>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I302" t="inlineStr"/>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>Generation Development</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr"/>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>Denver, CO</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>Condo developer; 1717 Washington Condos (Marieta)</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/project-portal/1717-washington-condos-uptown</t>
+        </is>
+      </c>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I303" t="inlineStr"/>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>Milwaukee Development LLC</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr"/>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>Denver, CO</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>55 N. Corona Townhomes</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/55-corona-townhomes-denver</t>
+        </is>
+      </c>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>March 2026</t>
+        </is>
+      </c>
+      <c r="I304" t="inlineStr"/>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>Golub &amp; Company</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr"/>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>Chicago, IL / Denver, CO</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>Denargo Market Building 1 (with Formativ)</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/denargo-market-16-story-site-development-plan</t>
+        </is>
+      </c>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>December 2025</t>
+        </is>
+      </c>
+      <c r="I305" t="inlineStr"/>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>Formativ</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr"/>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>Denver, CO</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>Denargo Market Building 1 (with Golub &amp; Company)</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/denargo-market-16-story-site-development-plan</t>
+        </is>
+      </c>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>December 2025</t>
+        </is>
+      </c>
+      <c r="I306" t="inlineStr"/>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>HLW International</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Architect</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>https://www.hlw.com</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>Architect for High Fidelity Plaza office-to-residential conversion</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/621-633-17th-street-office-to-residential-conversion-denver</t>
+        </is>
+      </c>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I307" t="inlineStr"/>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>Bryant Flink Architecture</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>Architect</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr"/>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>Denver, CO</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>Architect for 1717 Washington Condos</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/project-portal/1717-washington-condos-uptown</t>
+        </is>
+      </c>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I308" t="inlineStr"/>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>Points West Design</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>Architect</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr"/>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>Denver, CO</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>Architect for 55 N. Corona Townhomes</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/55-corona-townhomes-denver</t>
+        </is>
+      </c>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>March 2026</t>
+        </is>
+      </c>
+      <c r="I309" t="inlineStr"/>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>Goettsch Partners</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>Architect</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>https://www.goettsch.com</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>Chicago, IL</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>Architect for Denargo Market Building 1</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/denargo-market-16-story-site-development-plan</t>
+        </is>
+      </c>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>December 2025</t>
+        </is>
+      </c>
+      <c r="I310" t="inlineStr"/>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>RIOS</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>Architect</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>https://www.rios.com</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>Los Angeles, CA</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>Landscape/Design architect for Skyline Park Redesign</t>
+        </is>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/closer-look-at-downtown-denvers-massive-skyline-park-transformation</t>
+        </is>
+      </c>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I311" t="inlineStr"/>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>Studio Gang</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>Architect</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>https://studiogang.com</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>Chicago, IL</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>Architect for Civic Center Park Next 100 renovation</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/civic-center-park-renovation-denver-next-100</t>
+        </is>
+      </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I312" t="inlineStr"/>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>HDR</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>Architect</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>https://www.hdrinc.com</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>Omaha, NE (Denver office)</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>Architect for Swansea Rec Center Indoor Pool</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/swansea-recreation-center-new-indoor-pool-denver</t>
+        </is>
+      </c>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="I313" t="inlineStr"/>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>Steele Properties</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr"/>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>Denver, CO</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>Co-developer on 602 W. 29th Ave affordable housing</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/70-unit-affordable-housing-29th-fox-denver</t>
+        </is>
+      </c>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I314" t="inlineStr"/>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>Sasaki</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>Landscape Architect</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>https://www.sasaki.com</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>Boston, MA (Denver projects)</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>Landscape architect for Denargo Market; Park Hill Park planner</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/denargo-market-16-story-site-development-plan</t>
+        </is>
+      </c>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I315" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -25024,7 +27302,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F128"/>
+  <dimension ref="A1:F146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -29131,6 +31409,582 @@
         </is>
       </c>
     </row>
+    <row r="129">
+      <c r="A129" s="3" t="inlineStr">
+        <is>
+          <t>The Luzzatto Company</t>
+        </is>
+      </c>
+      <c r="B129" s="3" t="inlineStr">
+        <is>
+          <t>High Fidelity Plaza</t>
+        </is>
+      </c>
+      <c r="C129" s="3" t="inlineStr">
+        <is>
+          <t>621-633 17th Street, Denver</t>
+        </is>
+      </c>
+      <c r="D129" s="3" t="inlineStr">
+        <is>
+          <t>Multifamily / Office-to-Residential</t>
+        </is>
+      </c>
+      <c r="E129" s="3" t="inlineStr">
+        <is>
+          <t>Proposed / Financing Approved</t>
+        </is>
+      </c>
+      <c r="F129" s="3" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/621-633-17th-street-office-to-residential-conversion-denver</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>The Luzzatto Company</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>Denver Energy Center Conversion</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
+          <t>1625 Broadway (Tower 2), Denver</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t>Multifamily / Office-to-Residential</t>
+        </is>
+      </c>
+      <c r="E130" s="2" t="inlineStr">
+        <is>
+          <t>Proposed (Concept Plan)</t>
+        </is>
+      </c>
+      <c r="F130" s="2" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/625-broadway-denver-energy-center-office-to-residential-conversion</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="3" t="inlineStr">
+        <is>
+          <t>Ulysses Development Group</t>
+        </is>
+      </c>
+      <c r="B131" s="3" t="inlineStr">
+        <is>
+          <t>Central Park Station Affordable Housing</t>
+        </is>
+      </c>
+      <c r="C131" s="3" t="inlineStr">
+        <is>
+          <t>3801 Ulster Street, Denver</t>
+        </is>
+      </c>
+      <c r="D131" s="3" t="inlineStr">
+        <is>
+          <t>Affordable Multifamily + Childcare – 150 units</t>
+        </is>
+      </c>
+      <c r="E131" s="3" t="inlineStr">
+        <is>
+          <t>Proposed (Concept Approved)</t>
+        </is>
+      </c>
+      <c r="F131" s="3" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/rtd-central-park-station-advances-150-unit-affordable-housing-project</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>Elevation Development Group</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>602 W. 29th Ave Affordable Housing</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr">
+        <is>
+          <t>602 West 29th Avenue, Denver</t>
+        </is>
+      </c>
+      <c r="D132" s="2" t="inlineStr">
+        <is>
+          <t>Affordable Multifamily – 70 units</t>
+        </is>
+      </c>
+      <c r="E132" s="2" t="inlineStr">
+        <is>
+          <t>Proposed (Concept Plan)</t>
+        </is>
+      </c>
+      <c r="F132" s="2" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/70-unit-affordable-housing-29th-fox-denver</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="3" t="inlineStr">
+        <is>
+          <t>Mile High Development</t>
+        </is>
+      </c>
+      <c r="B133" s="3" t="inlineStr">
+        <is>
+          <t>University Building Affordable Housing</t>
+        </is>
+      </c>
+      <c r="C133" s="3" t="inlineStr">
+        <is>
+          <t>910 16th Street, Denver</t>
+        </is>
+      </c>
+      <c r="D133" s="3" t="inlineStr">
+        <is>
+          <t>Affordable Multifamily / Office-to-Residential</t>
+        </is>
+      </c>
+      <c r="E133" s="3" t="inlineStr">
+        <is>
+          <t>Proposed (Concept Plan Resubmitted)</t>
+        </is>
+      </c>
+      <c r="F133" s="3" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/university-building-affordable-housing-denver</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>BB Living</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>Northfield Duplex Community</t>
+        </is>
+      </c>
+      <c r="C134" s="2" t="inlineStr">
+        <is>
+          <t>8510 Northfield Boulevard, Denver</t>
+        </is>
+      </c>
+      <c r="D134" s="2" t="inlineStr">
+        <is>
+          <t>For-Rent Duplex – 210 units</t>
+        </is>
+      </c>
+      <c r="E134" s="2" t="inlineStr">
+        <is>
+          <t>Proposed (Concept Plan)</t>
+        </is>
+      </c>
+      <c r="F134" s="2" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/northfield-denver-210-unit-duplex-development</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="3" t="inlineStr">
+        <is>
+          <t>Generation Development</t>
+        </is>
+      </c>
+      <c r="B135" s="3" t="inlineStr">
+        <is>
+          <t>Marieta / 1717 Washington Condos</t>
+        </is>
+      </c>
+      <c r="C135" s="3" t="inlineStr">
+        <is>
+          <t>1717 N. Washington Street, Denver</t>
+        </is>
+      </c>
+      <c r="D135" s="3" t="inlineStr">
+        <is>
+          <t>Condos + Retail</t>
+        </is>
+      </c>
+      <c r="E135" s="3" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
+      <c r="F135" s="3" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/project-portal/1717-washington-condos-uptown</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>Golub &amp; Company</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>Denargo Market – Building 1</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t>Denargo St &amp; Delgany St, Denver (RiNo)</t>
+        </is>
+      </c>
+      <c r="D136" s="2" t="inlineStr">
+        <is>
+          <t>Mixed-Use – 16-story</t>
+        </is>
+      </c>
+      <c r="E136" s="2" t="inlineStr">
+        <is>
+          <t>Under Review / SDP Filed</t>
+        </is>
+      </c>
+      <c r="F136" s="2" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/denargo-market-16-story-site-development-plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="3" t="inlineStr">
+        <is>
+          <t>City of Denver</t>
+        </is>
+      </c>
+      <c r="B137" s="3" t="inlineStr">
+        <is>
+          <t>Civic Center Next 100</t>
+        </is>
+      </c>
+      <c r="C137" s="3" t="inlineStr">
+        <is>
+          <t>Civic Center Park, Denver</t>
+        </is>
+      </c>
+      <c r="D137" s="3" t="inlineStr">
+        <is>
+          <t>Parks / Public Space Renovation</t>
+        </is>
+      </c>
+      <c r="E137" s="3" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
+      <c r="F137" s="3" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/civic-center-park-renovation-denver-next-100</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>City of Denver</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>Skyline Park Redesign</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t>Arapahoe St between 16th &amp; 17th St, Denver</t>
+        </is>
+      </c>
+      <c r="D138" s="2" t="inlineStr">
+        <is>
+          <t>Parks / Public Space Redesign</t>
+        </is>
+      </c>
+      <c r="E138" s="2" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
+      <c r="F138" s="2" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/closer-look-at-downtown-denvers-massive-skyline-park-transformation</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="3" t="inlineStr">
+        <is>
+          <t>City of Denver</t>
+        </is>
+      </c>
+      <c r="B139" s="3" t="inlineStr">
+        <is>
+          <t>Swansea Recreation Center Indoor Pool</t>
+        </is>
+      </c>
+      <c r="C139" s="3" t="inlineStr">
+        <is>
+          <t>2581 Valentia St, Denver</t>
+        </is>
+      </c>
+      <c r="D139" s="3" t="inlineStr">
+        <is>
+          <t>Public Aquatic Facility</t>
+        </is>
+      </c>
+      <c r="E139" s="3" t="inlineStr">
+        <is>
+          <t>Completed / Opened May 2026</t>
+        </is>
+      </c>
+      <c r="F139" s="3" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/swansea-recreation-center-new-indoor-pool-denver</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>Denver Museum of Nature &amp; Science</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>Gems &amp; Minerals Hall Renovation</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>2001 Colorado Blvd, Denver</t>
+        </is>
+      </c>
+      <c r="D140" s="2" t="inlineStr">
+        <is>
+          <t>Museum Renovation – $30M</t>
+        </is>
+      </c>
+      <c r="E140" s="2" t="inlineStr">
+        <is>
+          <t>Under Construction; closed 2026</t>
+        </is>
+      </c>
+      <c r="F140" s="2" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/denver-museum-gems-minerals-hall-renovation-30m-closure-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="3" t="inlineStr">
+        <is>
+          <t>Milwaukee Development LLC</t>
+        </is>
+      </c>
+      <c r="B141" s="3" t="inlineStr">
+        <is>
+          <t>55 N. Corona Townhomes</t>
+        </is>
+      </c>
+      <c r="C141" s="3" t="inlineStr">
+        <is>
+          <t>55 N. Corona Street, Denver</t>
+        </is>
+      </c>
+      <c r="D141" s="3" t="inlineStr">
+        <is>
+          <t>Residential Townhomes</t>
+        </is>
+      </c>
+      <c r="E141" s="3" t="inlineStr">
+        <is>
+          <t>Proposed (Concept Plan)</t>
+        </is>
+      </c>
+      <c r="F141" s="3" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/55-corona-townhomes-denver</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>Matthew Lawrence / John Crays</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>The Berg at Shoenberg Farms</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>73rd Ave &amp; Sheridan Blvd, Westminster</t>
+        </is>
+      </c>
+      <c r="D142" s="2" t="inlineStr">
+        <is>
+          <t>Food Hall / Entertainment / Retail</t>
+        </is>
+      </c>
+      <c r="E142" s="2" t="inlineStr">
+        <is>
+          <t>Proposed / Under Development</t>
+        </is>
+      </c>
+      <c r="F142" s="2" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/the-berg-shoenberg-farms-westminster-food-hall</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="3" t="inlineStr">
+        <is>
+          <t>FCI Constructors</t>
+        </is>
+      </c>
+      <c r="B143" s="3" t="inlineStr">
+        <is>
+          <t>Swansea Rec Center Indoor Pool (GC)</t>
+        </is>
+      </c>
+      <c r="C143" s="3" t="inlineStr">
+        <is>
+          <t>2581 Valentia St, Denver</t>
+        </is>
+      </c>
+      <c r="D143" s="3" t="inlineStr">
+        <is>
+          <t>Public Aquatic Facility</t>
+        </is>
+      </c>
+      <c r="E143" s="3" t="inlineStr">
+        <is>
+          <t>Completed / Opened May 2026</t>
+        </is>
+      </c>
+      <c r="F143" s="3" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/swansea-recreation-center-new-indoor-pool-denver</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>SAR+ Architects</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>Central Park Station Affordable Housing</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>3801 Ulster Street, Denver</t>
+        </is>
+      </c>
+      <c r="D144" s="2" t="inlineStr">
+        <is>
+          <t>Affordable Multifamily – Architecture</t>
+        </is>
+      </c>
+      <c r="E144" s="2" t="inlineStr">
+        <is>
+          <t>Proposed (Concept Approved)</t>
+        </is>
+      </c>
+      <c r="F144" s="2" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/rtd-central-park-station-advances-150-unit-affordable-housing-project</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="3" t="inlineStr">
+        <is>
+          <t>Semple Brown Design</t>
+        </is>
+      </c>
+      <c r="B145" s="3" t="inlineStr">
+        <is>
+          <t>The James</t>
+        </is>
+      </c>
+      <c r="C145" s="3" t="inlineStr">
+        <is>
+          <t>Evans Ave &amp; S. Gilpin St, Denver</t>
+        </is>
+      </c>
+      <c r="D145" s="3" t="inlineStr">
+        <is>
+          <t>Mixed-Use Multifamily – Architecture</t>
+        </is>
+      </c>
+      <c r="E145" s="3" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
+      <c r="F145" s="3" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/the-james-evans-gilpin-denver</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>Goettsch Partners</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>Denargo Market – Building 1</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>Denargo St &amp; Delgany St, Denver (RiNo)</t>
+        </is>
+      </c>
+      <c r="D146" s="2" t="inlineStr">
+        <is>
+          <t>Mixed-Use – 16-story – Architecture</t>
+        </is>
+      </c>
+      <c r="E146" s="2" t="inlineStr">
+        <is>
+          <t>Under Review / SDP Filed</t>
+        </is>
+      </c>
+      <c r="F146" s="2" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/denargo-market-16-story-site-development-plan</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:F120"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Deep scrape developingmycity.com: +32 projects, +31 companies, +4 contacts, +20 current projects
Exhaustive site: search across 30+ neighborhood/type combinations surfaced
56 unique articles. Added Broadway Station Block 1, Rock Drill RiNo ($585M),
Broncos Burnham Yard proposal, Four Seasons Cherry Creek, National Western
Center expansion, ACE Padel RiNo, Barth Hotel Senior Housing, and more.

https://claude.ai/code/session_016XhpERgAeaSiATUKTdFgci
</commit_message>
<xml_diff>
--- a/Naked_Denver_Contact_Directory_Combined.xlsx
+++ b/Naked_Denver_Contact_Directory_Combined.xlsx
@@ -623,7 +623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I89"/>
+  <dimension ref="A1:I121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4806,6 +4806,1510 @@
       <c r="I89" t="inlineStr">
         <is>
           <t>https://www.developingmycity.com/denver/news/64-unit-townhome-project-northeast-denver-dillon-street</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Barth Hotel Senior Housing</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>1514 17th Street, Denver</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Downtown / LoDo</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/barth-hotel-senior-housing-concept-1514-17th-denver</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Concept Plan; $6M DDDA loan approved Jan 2026</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>50-unit affordable senior housing (30-50% AMI), 4-story historic adaptive reuse. Developer: Senior Housing Options Inc. / Urban Ventures / Eaton Senior. Architect: Shopworks Architecture.</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Jan 2026</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/barth-hotel-senior-housing-concept-1514-17th-denver</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>University Hills Rowhomes</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>S Ivanhoe St &amp; E Jefferson Ave, Denver</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>University Hills</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/university-hills-rowhome-development-ivanhoe</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Proposed (Concept Plan)</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>75 rowhomes + 7 SFR.</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>~2025</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/university-hills-rowhome-development-ivanhoe</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>South Federal Mixed-Use</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>South Federal Blvd &amp; W Tennessee Ave, Denver</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Southwest Denver</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/south-federal-mixed-use-development-denver-99-units</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Under Community Review</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>99 units + 30,000 SF retail, 4-story mixed-use.</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Apr 24 2026</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/south-federal-mixed-use-development-denver-99-units</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Holiday Inn Conversion – 240 Units</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>3333 N Quebec Street, Denver</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Northeast Denver / Stapleton</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/holiday-inn-3333-n-quebec-240-unit-apartment-conversion-approved</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Concept Plan Approved / Advancing to SDP</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>240-unit, 11-story adaptive reuse of Holiday Inn. Developer: Eagle Propco 7 LLC / Premier Project Management.</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>~2025</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/holiday-inn-3333-n-quebec-240-unit-apartment-conversion-approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Broadway Station Block 1</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Broadway Station, South Denver</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>South Denver / Broadway Corridor</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/7-story-residential-project-planned-for-broadway-station-block-1</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>SDP Review In Progress</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>367 units, 7-story + public plaza. Developer: Santa Fe Denver G LLC. Architect: Davis Partnership. Civil: Kimley-Horn.</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>~2025</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/7-story-residential-project-planned-for-broadway-station-block-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>6-Unit Townhomes Near DU</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Near University of Denver, Denver</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>University</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/6-unit-townhome-development-near-university-of-denver</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>SDP Filed</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>6-unit townhomes.</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>~2025</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/6-unit-townhome-development-near-university-of-denver</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>ACE Padel RiNo</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>1812 35th Street, Denver</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>RiNo</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/ace-padel-rino-concept-plan-approved</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Concept Plan Approved</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>5 indoor + 3 outdoor padel courts, bar. Developer: ACE Padel / Aventura Asset Management. Architect: Roth Sheppard.</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>~2026</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/ace-padel-rino-concept-plan-approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Denver First Common Consumption Area – Mission Ballroom</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>4180 Wynkoop Street, Denver</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>RiNo</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/denver-first-common-consumption-area-rino</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Approved by City Council Jan 2026</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Denver's first common consumption area (outdoor alcohol). Owner: Westfield Company Inc.</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Jan 2026</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/denver-first-common-consumption-area-rino</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Hopscotch Beer Garden – Denargo Market</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>3380 Denargo Street, Denver</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>RiNo</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/hopscotch-beer-garden-approved-for-denargo-market-opening-planned-for-2026</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Approved; Opening late winter 2026</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>17,000 SF food &amp; beverage / outdoor beer garden. Developer: Golub &amp; Company / FORMATIV. Operator: DrinkDenver.</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>~2026</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/hopscotch-beer-garden-approved-for-denargo-market-opening-planned-for-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Kensing LoHi Condos</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>1643 Boulder Street, Denver</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>LoHi</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/kensing-lohi-condos-denver-lower-highlands</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Nearing Completion / Grand Opening Jun 2026</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>35 for-sale condos. Developer: Urban Green Development. Architects: Neo Studio / Coesivo Design Group.</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>~2026</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/kensing-lohi-condos-denver-lower-highlands</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Sloan's Lake Boathouse Renovation</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Sloan's Lake Park, Denver</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Sloan's Lake</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/sloans-lake-boathouse-renovation-preferred-design</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Preferred Design Concept Released</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>$7M recreation / community space renovation. Architect: Studio Gang.</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>~2025</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/sloans-lake-boathouse-renovation-preferred-design</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Park Avenue Apartments – Globeville</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>3721 N Globeville Road, Denver</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Globeville</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/park-avenue-apartments-globeville-supportive-housing</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Under Construction (financing closed)</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>60-unit supportive housing, adaptive reuse of La Quinta hotel. Developer: Colorado Coalition for the Homeless (CCH). Architect: Davis Partnership Architects.</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>~2025</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/park-avenue-apartments-globeville-supportive-housing</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Paragon Place – Supportive Housing</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>2205 N Washington Street, Denver</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Five Points</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/paragon-place-supportive-housing-2205-washington-denver</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Concept Plan Filed</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>55 units + nonprofit space, 4-story supportive housing.</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>~2025</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/paragon-place-supportive-housing-2205-washington-denver</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>1139 Delaware – Supportive Housing</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>1139 Delaware Street, Denver</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Golden Triangle</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/1139-delaware-supportive-housing-renderings</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Under Review</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>80-unit, 6-story supportive housing. Developer: Denver Housing Authority (DHA). Architect: KTGY.</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>~2025</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/1139-delaware-supportive-housing-renderings</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>135-Unit Affordable Housing – 40th &amp; York</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>SE corner E 40th Ave &amp; York Street, Denver</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Cole / RiNo Adjacent</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/40th-york-affordable-housing-concept-plan</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Concept Plan (Intake in Progress)</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>135 units, 4-story, 100% income-restricted. Developer: RH Group. Architect: KTGY. Civil: Kimley-Horn.</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Jan 2026</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/40th-york-affordable-housing-concept-plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>125-Unit Affordable Housing – North Federal / Rocky Mountain Lake</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>4745 N Federal Boulevard, Denver</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Northwest Denver</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/north-federal-affordable-housing-cch-rocky-mountain-lake</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Concept Review / Prop 123 Fast-Track</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>125 units: 40 supportive + 85 family + daycare. Developer: Colorado Coalition for the Homeless / Denver Housing Authority (ground lease).</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Feb/Mar 2026</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/north-federal-affordable-housing-cch-rocky-mountain-lake</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Denver Broncos – Burnham Yard Stadium</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Burnham Yard, ~10th &amp; Osage, Denver</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Lincoln Park / Sun Valley</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/denver-broncos-burnham-yard-stadium-proposal-community-meeting</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Rezoning / Early Planning</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>150-acre stadium + mixed-use district. Developer: Denver Broncos. Master planner: Sasaki. Small area planner: Perkins&amp;Will.</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>~2025-2026</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/denver-broncos-burnham-yard-stadium-proposal-community-meeting</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>11-Story Mixed-Use Near Ball Arena</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Near Ball Arena, Denver</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Central Platte Valley</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/11-story-concept-parking-lot-near-ball-arena</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Concept Submitted</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>11-story mixed-use on parking lot near Ball Arena.</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>~2025</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/11-story-concept-parking-lot-near-ball-arena</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>National Western Center $185M Expansion</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>National Western Center campus, Denver</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Elyria-Swansea / Globeville</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/national-western-center-185m-expansion</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>SDP Filed</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>726,000 SF equestrian complex + 9-story hotel + parking, $185M.</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>~2025</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/national-western-center-185m-expansion</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Crunch Fitness – Hampden</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>7400 E Hampden Avenue, Denver</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Southeast Denver</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/crunch-fitness-hampden-avenue-denver-concept-plan</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Concept Plan Filed</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Commercial fitness remodel. Architect: JPLUS Architects Inc.</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>~2025</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/crunch-fitness-hampden-avenue-denver-concept-plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Link 56 – Parcel H Retail</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>E 56th Ave &amp; Tower Road, Denver (Gateway/Near DIA)</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Gateway / Near DIA</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/link-56-parcel-h-retail-building-designs</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Concept Plan / Design Revealed</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>2 retail buildings, 6,500 SF. Developer: Kensington Development Partners. Architect: Galloway &amp; Company.</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>~2025</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/link-56-parcel-h-retail-building-designs</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Elevate Travel Center – DIA</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>S of Peña Blvd, Denver (near DIA)</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Near DIA</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/elevate-travel-center-breaks-ground-near-denver-international-airport</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Under Construction; completion Summer 2026</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Travel convenience center: fueling, car wash, EV charging, retail. Developer: Aaravya Investments / DEN. Architect: Paragon4Design.</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>~2025</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/elevate-travel-center-breaks-ground-near-denver-international-airport</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>DIA Concourse Walkways</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Denver International Airport, Denver</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Near DIA</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/denver-international-airport-confirms-new-concourse-walkways</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Announced; construction ~2027</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>New pedestrian walkways connecting Concourses A-B-C.</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>~2025</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/denver-international-airport-confirms-new-concourse-walkways</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Brookfield Contour Townhomes – Central Park</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>E 47th Ave &amp; Beeler Court, Denver</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Central Park</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/brookfield-contour-townhomes-central-park-denver</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Under Construction / New Phase</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>3-level, 2-3BR townhomes. Developer: Brookfield Residential.</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>Apr 17 2026</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/brookfield-contour-townhomes-central-park-denver</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>17-Unit Townhomes – W 13th Ave</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>4862 W 13th Avenue, Denver</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>West Denver</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/west-13th-avenue-townhomes-denver-17-units</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>17 units, 3 buildings, 3-story.</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>~2025</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/west-13th-avenue-townhomes-denver-17-units</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>368-Unit Multifamily – South Havana</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>6901 S Havana Street, Centennial</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Centennial (Denver Metro)</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/centennial-south-havana-multifamily-368-units</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>368 units, 14 buildings. Developer: Buchanan Capital Partners / The Garrett Companies. Architect: Ware Malcomb.</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>~2025</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/centennial-south-havana-multifamily-368-units</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Four Seasons Private Residences – Cherry Creek</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>215-231 N Detroit Street, Denver</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Cherry Creek North</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/four-seasons-condos-cherry-creek-detroit-street</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Urban Design Review (filed Jan 2026)</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>41-42 luxury condos, 8-story. Developer: Stillwater Capital / Wexford Real Estate Investors / Brue Baukol Capital Partners / Zabel Investment Co.</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>Jan/Feb 2026</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/four-seasons-condos-cherry-creek-detroit-street</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Cherry Creek West – Zone Lot A Office</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>1st Ave &amp; Road H, Denver</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Cherry Creek West</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/cherry-creek-west-zone-lot-a-site-design-massing</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Site Design &amp; Massing Filed</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>8-story office/retail as part of Cherry Creek West. Developer: East West Partners. GC: Mortenson/Saunders JV. Architects: Gensler / GBD / Design Workshop.</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>~2025-2026</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/cherry-creek-west-zone-lot-a-site-design-massing</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Rock Drill RiNo Redevelopment</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>1717 E 39th Avenue, Denver (6.7-acre site)</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Cole / RiNo</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/tag/Mixed-Use+Development</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Rezoning / TIF Financing Under Review</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>$585M mixed-use: housing, retail, office, hotel. Developer: OliverBuchanan Group / Weiss Family.</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>~2025</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/tag/Mixed-Use+Development</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Historic Nurses Dorm – 9th+Colorado</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>4200 E 9th Avenue, Denver</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Hale / 9th+Colorado</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/historic-nurses-dorm-9th-colorado-wellness-redevelopment</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Concept Plan Filed</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>25,000-27,000 SF medical office / wellness / coworking, adaptive reuse. Developer: Continuum Partners.</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>~2025</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/historic-nurses-dorm-9th-colorado-wellness-redevelopment</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>1415 Tremont Place Adaptive Reuse</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>1415 Tremont Place, Denver</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Downtown / CBD</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/tag/CBD</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Concept Plan</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>2-story, 9,000 SF office/retail/childcare. Developer: Kippah LLC.</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>~2025</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/tag/CBD</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Valverde Mixed-Use</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>2100 W Alameda Avenue, Denver</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Valverde</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/project-portal</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Formal SDP</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>26 apts + 10,000 SF retail, 3-story, 65,000 SF.</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>~2025</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/project-portal</t>
         </is>
       </c>
     </row>
@@ -4820,7 +6324,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M177"/>
+  <dimension ref="A1:M181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13843,9 +15347,6 @@
           <t>President</t>
         </is>
       </c>
-      <c r="F168" t="inlineStr"/>
-      <c r="G168" t="inlineStr"/>
-      <c r="H168" t="inlineStr"/>
       <c r="I168" t="inlineStr">
         <is>
           <t>https://www.developingmycity.com/denver/news/621-633-17th-street-office-to-residential-conversion-denver</t>
@@ -13866,7 +15367,6 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="M168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -13894,9 +15394,6 @@
           <t>Managing Partner</t>
         </is>
       </c>
-      <c r="F169" t="inlineStr"/>
-      <c r="G169" t="inlineStr"/>
-      <c r="H169" t="inlineStr"/>
       <c r="I169" t="inlineStr">
         <is>
           <t>https://www.developingmycity.com/denver/news/rtd-central-park-station-advances-150-unit-affordable-housing-project</t>
@@ -13917,7 +15414,6 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="M169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -13945,9 +15441,6 @@
           <t>Founding Partner &amp; CEO</t>
         </is>
       </c>
-      <c r="F170" t="inlineStr"/>
-      <c r="G170" t="inlineStr"/>
-      <c r="H170" t="inlineStr"/>
       <c r="I170" t="inlineStr">
         <is>
           <t>https://www.developingmycity.com/denver/news/university-building-affordable-housing-denver</t>
@@ -13968,7 +15461,6 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="M170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -13996,9 +15488,6 @@
           <t>Principal</t>
         </is>
       </c>
-      <c r="F171" t="inlineStr"/>
-      <c r="G171" t="inlineStr"/>
-      <c r="H171" t="inlineStr"/>
       <c r="I171" t="inlineStr">
         <is>
           <t>https://www.developingmycity.com/denver/news/university-building-affordable-housing-denver</t>
@@ -14019,7 +15508,6 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="M171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -14047,9 +15535,6 @@
           <t>President</t>
         </is>
       </c>
-      <c r="F172" t="inlineStr"/>
-      <c r="G172" t="inlineStr"/>
-      <c r="H172" t="inlineStr"/>
       <c r="I172" t="inlineStr">
         <is>
           <t>https://www.developingmycity.com/denver/project-portal/1717-washington-condos-uptown</t>
@@ -14070,7 +15555,6 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="M172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -14098,9 +15582,6 @@
           <t>Partner</t>
         </is>
       </c>
-      <c r="F173" t="inlineStr"/>
-      <c r="G173" t="inlineStr"/>
-      <c r="H173" t="inlineStr"/>
       <c r="I173" t="inlineStr">
         <is>
           <t>https://www.developingmycity.com/denver/news/70-unit-affordable-housing-29th-fox-denver</t>
@@ -14121,7 +15602,6 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="M173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -14149,9 +15629,6 @@
           <t>Founder</t>
         </is>
       </c>
-      <c r="F174" t="inlineStr"/>
-      <c r="G174" t="inlineStr"/>
-      <c r="H174" t="inlineStr"/>
       <c r="I174" t="inlineStr">
         <is>
           <t>https://www.developingmycity.com/denver/news/70-unit-affordable-housing-29th-fox-denver</t>
@@ -14172,7 +15649,6 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="M174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -14200,9 +15676,6 @@
           <t>Partner</t>
         </is>
       </c>
-      <c r="F175" t="inlineStr"/>
-      <c r="G175" t="inlineStr"/>
-      <c r="H175" t="inlineStr"/>
       <c r="I175" t="inlineStr">
         <is>
           <t>https://www.developingmycity.com/denver/news/70-unit-affordable-housing-29th-fox-denver</t>
@@ -14223,7 +15696,6 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="M175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -14251,9 +15723,6 @@
           <t>Developer/Co-owner</t>
         </is>
       </c>
-      <c r="F176" t="inlineStr"/>
-      <c r="G176" t="inlineStr"/>
-      <c r="H176" t="inlineStr"/>
       <c r="I176" t="inlineStr">
         <is>
           <t>https://www.developingmycity.com/denver/news/the-berg-shoenberg-farms-westminster-food-hall</t>
@@ -14274,7 +15743,6 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="M176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -14302,9 +15770,6 @@
           <t>Developer/Co-owner</t>
         </is>
       </c>
-      <c r="F177" t="inlineStr"/>
-      <c r="G177" t="inlineStr"/>
-      <c r="H177" t="inlineStr"/>
       <c r="I177" t="inlineStr">
         <is>
           <t>https://www.developingmycity.com/denver/news/the-berg-shoenberg-farms-westminster-food-hall</t>
@@ -14325,7 +15790,210 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="M177" t="inlineStr"/>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Rock Drill RiNo Redevelopment</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>OliverBuchanan Group</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Morgan Dene Oliver</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>Chairman</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr"/>
+      <c r="G178" t="inlineStr"/>
+      <c r="H178" t="inlineStr"/>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/tag/Mixed-Use+Development</t>
+        </is>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="M178" t="inlineStr"/>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Rock Drill RiNo Redevelopment</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>OliverBuchanan Group</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Eric Buchanan</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr"/>
+      <c r="G179" t="inlineStr"/>
+      <c r="H179" t="inlineStr"/>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/tag/Mixed-Use+Development</t>
+        </is>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="L179" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="M179" t="inlineStr"/>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>ACE Padel RiNo</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>ACE Padel</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Operator</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Peter Carnello</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr"/>
+      <c r="G180" t="inlineStr"/>
+      <c r="H180" t="inlineStr"/>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/ace-padel-rino-concept-plan-approved</t>
+        </is>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="M180" t="inlineStr"/>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>ACE Padel RiNo</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>ACE Padel</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Operator</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Elliot Carnello</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr"/>
+      <c r="G181" t="inlineStr"/>
+      <c r="H181" t="inlineStr"/>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/ace-padel-rino-concept-plan-approved</t>
+        </is>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="M181" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -14338,7 +16006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I315"/>
+  <dimension ref="A1:I346"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26353,7 +28021,6 @@
           <t>Developer</t>
         </is>
       </c>
-      <c r="C299" t="inlineStr"/>
       <c r="D299" t="inlineStr">
         <is>
           <t>New York, NY</t>
@@ -26379,7 +28046,6 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="I299" t="inlineStr"/>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -26392,7 +28058,6 @@
           <t>Developer</t>
         </is>
       </c>
-      <c r="C300" t="inlineStr"/>
       <c r="D300" t="inlineStr">
         <is>
           <t>Denver, CO</t>
@@ -26418,7 +28083,6 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="I300" t="inlineStr"/>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -26431,7 +28095,6 @@
           <t>Developer</t>
         </is>
       </c>
-      <c r="C301" t="inlineStr"/>
       <c r="D301" t="inlineStr">
         <is>
           <t>Denver, CO</t>
@@ -26457,7 +28120,6 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="I301" t="inlineStr"/>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -26470,7 +28132,6 @@
           <t>Developer</t>
         </is>
       </c>
-      <c r="C302" t="inlineStr"/>
       <c r="D302" t="inlineStr">
         <is>
           <t>Denver, CO</t>
@@ -26496,7 +28157,6 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="I302" t="inlineStr"/>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -26509,7 +28169,6 @@
           <t>Developer</t>
         </is>
       </c>
-      <c r="C303" t="inlineStr"/>
       <c r="D303" t="inlineStr">
         <is>
           <t>Denver, CO</t>
@@ -26535,7 +28194,6 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="I303" t="inlineStr"/>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -26548,7 +28206,6 @@
           <t>Developer</t>
         </is>
       </c>
-      <c r="C304" t="inlineStr"/>
       <c r="D304" t="inlineStr">
         <is>
           <t>Denver, CO</t>
@@ -26574,7 +28231,6 @@
           <t>March 2026</t>
         </is>
       </c>
-      <c r="I304" t="inlineStr"/>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -26587,7 +28243,6 @@
           <t>Developer</t>
         </is>
       </c>
-      <c r="C305" t="inlineStr"/>
       <c r="D305" t="inlineStr">
         <is>
           <t>Chicago, IL / Denver, CO</t>
@@ -26613,7 +28268,6 @@
           <t>December 2025</t>
         </is>
       </c>
-      <c r="I305" t="inlineStr"/>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -26626,7 +28280,6 @@
           <t>Developer</t>
         </is>
       </c>
-      <c r="C306" t="inlineStr"/>
       <c r="D306" t="inlineStr">
         <is>
           <t>Denver, CO</t>
@@ -26652,7 +28305,6 @@
           <t>December 2025</t>
         </is>
       </c>
-      <c r="I306" t="inlineStr"/>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -26695,7 +28347,6 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="I307" t="inlineStr"/>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -26708,7 +28359,6 @@
           <t>Architect</t>
         </is>
       </c>
-      <c r="C308" t="inlineStr"/>
       <c r="D308" t="inlineStr">
         <is>
           <t>Denver, CO</t>
@@ -26734,7 +28384,6 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="I308" t="inlineStr"/>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -26747,7 +28396,6 @@
           <t>Architect</t>
         </is>
       </c>
-      <c r="C309" t="inlineStr"/>
       <c r="D309" t="inlineStr">
         <is>
           <t>Denver, CO</t>
@@ -26773,7 +28421,6 @@
           <t>March 2026</t>
         </is>
       </c>
-      <c r="I309" t="inlineStr"/>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -26816,7 +28463,6 @@
           <t>December 2025</t>
         </is>
       </c>
-      <c r="I310" t="inlineStr"/>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -26859,7 +28505,6 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="I311" t="inlineStr"/>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -26902,7 +28547,6 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="I312" t="inlineStr"/>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -26945,7 +28589,6 @@
           <t>May 2026</t>
         </is>
       </c>
-      <c r="I313" t="inlineStr"/>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
@@ -26958,7 +28601,6 @@
           <t>Developer</t>
         </is>
       </c>
-      <c r="C314" t="inlineStr"/>
       <c r="D314" t="inlineStr">
         <is>
           <t>Denver, CO</t>
@@ -26984,7 +28626,6 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="I314" t="inlineStr"/>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -27027,7 +28668,1199 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="I315" t="inlineStr"/>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>The Beck Group</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>General Contractor</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>https://www.beckgroup.com</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>Dallas, TX (Denver projects)</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>GC for Oasis Apartments, Cherry Creek</t>
+        </is>
+      </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/oasis-apartments-topping-out-299-milwaukee-cherry-creek</t>
+        </is>
+      </c>
+      <c r="G316" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I316" t="inlineStr"/>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>Senior Housing Options Inc.</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>Nonprofit / Developer</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr"/>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>Denver, CO</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>Owner/developer for Barth Hotel Senior Housing</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/barth-hotel-senior-housing-concept-1514-17th-denver</t>
+        </is>
+      </c>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I317" t="inlineStr"/>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>Urban Ventures</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr"/>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>Denver, CO</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>Co-developer for Barth Hotel Senior Housing</t>
+        </is>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/barth-hotel-senior-housing-concept-1514-17th-denver</t>
+        </is>
+      </c>
+      <c r="G318" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I318" t="inlineStr"/>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>Eaton Senior</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr"/>
+      <c r="D319" t="inlineStr"/>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>Co-developer for Barth Hotel Senior Housing</t>
+        </is>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/barth-hotel-senior-housing-concept-1514-17th-denver</t>
+        </is>
+      </c>
+      <c r="G319" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I319" t="inlineStr"/>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>MAA (Mid-America Apartment Communities)</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>Developer / REIT</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>https://www.maac.com</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>Memphis, TN</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>Developer for Milepost 35 Central Park (429 units)</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/429-unit-multifamily-development-central-park-denver</t>
+        </is>
+      </c>
+      <c r="G320" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I320" t="inlineStr"/>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>Eagle Propco 7 LLC</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>Owner / Developer</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr"/>
+      <c r="D321" t="inlineStr"/>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>Owner entity for Holiday Inn Conversion (3333 N Quebec, 240 units)</t>
+        </is>
+      </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/holiday-inn-3333-n-quebec-240-unit-apartment-conversion-approved</t>
+        </is>
+      </c>
+      <c r="G321" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H321" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I321" t="inlineStr"/>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>Premier Project Management</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>Property Manager</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr"/>
+      <c r="D322" t="inlineStr"/>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>Manager of record for Holiday Inn Conversion</t>
+        </is>
+      </c>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/holiday-inn-3333-n-quebec-240-unit-apartment-conversion-approved</t>
+        </is>
+      </c>
+      <c r="G322" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H322" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I322" t="inlineStr"/>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>Aventura Asset Management</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr"/>
+      <c r="D323" t="inlineStr"/>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>Development partner for ACE Padel RiNo</t>
+        </is>
+      </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/ace-padel-rino-concept-plan-approved</t>
+        </is>
+      </c>
+      <c r="G323" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I323" t="inlineStr"/>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>Roth Sheppard Architects</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>Architect</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>https://rothsheppard.com</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>Denver, CO</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>Architect for ACE Padel RiNo</t>
+        </is>
+      </c>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/ace-padel-rino-concept-plan-approved</t>
+        </is>
+      </c>
+      <c r="G324" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H324" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I324" t="inlineStr"/>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>Westfield Company Inc.</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>Property Owner</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr"/>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>Denver, CO</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>Owner of Mission Ballroom / Denver's first common consumption area</t>
+        </is>
+      </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/denver-first-common-consumption-area-rino</t>
+        </is>
+      </c>
+      <c r="G325" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H325" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I325" t="inlineStr"/>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>DrinkDenver</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>Food &amp; Beverage Operator</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr"/>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>Denver, CO</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>Operator for Hopscotch Beer Garden at Denargo Market</t>
+        </is>
+      </c>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/hopscotch-beer-garden-approved-for-denargo-market-opening-planned-for-2026</t>
+        </is>
+      </c>
+      <c r="G326" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H326" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I326" t="inlineStr"/>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>Urban Green Development</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr"/>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>Denver, CO</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>Developer for Kensing LoHi Condos</t>
+        </is>
+      </c>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/kensing-lohi-condos-denver-lower-highlands</t>
+        </is>
+      </c>
+      <c r="G327" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H327" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I327" t="inlineStr"/>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>Neo Studio</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>Architect</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr"/>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>Denver, CO</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>Design architect for Kensing LoHi Condos</t>
+        </is>
+      </c>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/kensing-lohi-condos-denver-lower-highlands</t>
+        </is>
+      </c>
+      <c r="G328" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H328" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I328" t="inlineStr"/>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>Coesivo Design Group</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>Architect</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr"/>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>Denver, CO</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>Design architect for Kensing LoHi Condos</t>
+        </is>
+      </c>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/kensing-lohi-condos-denver-lower-highlands</t>
+        </is>
+      </c>
+      <c r="G329" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H329" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I329" t="inlineStr"/>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>Denver Housing Authority</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>Public Developer</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>https://www.denverhousing.org</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>Denver, CO</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>Developer for 1139 Delaware supportive housing; ground lessor for North Federal CCH project</t>
+        </is>
+      </c>
+      <c r="F330" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/1139-delaware-supportive-housing-renderings</t>
+        </is>
+      </c>
+      <c r="G330" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H330" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I330" t="inlineStr"/>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>RH Group</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr"/>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>Denver, CO</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>Developer for 135-unit affordable housing at 40th &amp; York</t>
+        </is>
+      </c>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/40th-york-affordable-housing-concept-plan</t>
+        </is>
+      </c>
+      <c r="G331" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H331" t="inlineStr">
+        <is>
+          <t>Jan 2026</t>
+        </is>
+      </c>
+      <c r="I331" t="inlineStr"/>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>Santa Fe Denver G LLC</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>Owner / Developer</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr"/>
+      <c r="D332" t="inlineStr"/>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>Owner entity for Broadway Station Block 1 (367 units)</t>
+        </is>
+      </c>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/7-story-residential-project-planned-for-broadway-station-block-1</t>
+        </is>
+      </c>
+      <c r="G332" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H332" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I332" t="inlineStr"/>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>Kensington Development Partners</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr"/>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>Denver, CO</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>Developer for Link 56 mixed-use near DIA</t>
+        </is>
+      </c>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/link-56-parcel-h-retail-building-designs</t>
+        </is>
+      </c>
+      <c r="G333" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H333" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I333" t="inlineStr"/>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>Aaravya Investments</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>Developer / Operator</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr"/>
+      <c r="D334" t="inlineStr"/>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>Minority-owned developer for Elevate Travel Center near DIA</t>
+        </is>
+      </c>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/elevate-travel-center-breaks-ground-near-denver-international-airport</t>
+        </is>
+      </c>
+      <c r="G334" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H334" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I334" t="inlineStr"/>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>Stillwater Capital</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr"/>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>Dallas, TX</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>Lead developer for Four Seasons Private Residences Cherry Creek</t>
+        </is>
+      </c>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/four-seasons-condos-cherry-creek-detroit-street</t>
+        </is>
+      </c>
+      <c r="G335" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H335" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I335" t="inlineStr"/>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>Wexford Real Estate Investors</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>Investor</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr"/>
+      <c r="D336" t="inlineStr"/>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>Investor for Four Seasons Private Residences Cherry Creek</t>
+        </is>
+      </c>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/four-seasons-condos-cherry-creek-detroit-street</t>
+        </is>
+      </c>
+      <c r="G336" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H336" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I336" t="inlineStr"/>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>Zabel Investment Company</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>Investor</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr"/>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>Denver, CO</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>Investor for Four Seasons Private Residences Cherry Creek</t>
+        </is>
+      </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/four-seasons-condos-cherry-creek-detroit-street</t>
+        </is>
+      </c>
+      <c r="G337" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H337" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I337" t="inlineStr"/>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>Brue Baukol Capital Partners</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>Investor / Developer</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr"/>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>Denver, CO</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>Capital partner on Four Seasons Condos Cherry Creek and Milwaukee Place</t>
+        </is>
+      </c>
+      <c r="F338" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/four-seasons-condos-cherry-creek-detroit-street</t>
+        </is>
+      </c>
+      <c r="G338" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H338" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I338" t="inlineStr"/>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>Buchanan Capital Partners</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr"/>
+      <c r="D339" t="inlineStr"/>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>Developer for 368-unit multifamily Centennial S Havana</t>
+        </is>
+      </c>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/centennial-south-havana-multifamily-368-units</t>
+        </is>
+      </c>
+      <c r="G339" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H339" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I339" t="inlineStr"/>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>The Garrett Companies</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr"/>
+      <c r="D340" t="inlineStr"/>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>Co-developer for 368-unit multifamily Centennial S Havana</t>
+        </is>
+      </c>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/centennial-south-havana-multifamily-368-units</t>
+        </is>
+      </c>
+      <c r="G340" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H340" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I340" t="inlineStr"/>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>Ware Malcomb</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>Architect</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>https://www.waremalcomb.com</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>Irvine, CA (Denver office)</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>Architect for 368-unit Centennial S Havana multifamily</t>
+        </is>
+      </c>
+      <c r="F341" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/centennial-south-havana-multifamily-368-units</t>
+        </is>
+      </c>
+      <c r="G341" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H341" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I341" t="inlineStr"/>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>JPLUS Architects Inc.</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>Architect</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr"/>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>Denver, CO</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>Architect for Crunch Fitness Hampden</t>
+        </is>
+      </c>
+      <c r="F342" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/crunch-fitness-hampden-avenue-denver-concept-plan</t>
+        </is>
+      </c>
+      <c r="G342" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H342" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I342" t="inlineStr"/>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>Rockpoint</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>Capital Partner / Investor</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>https://www.rockpoint.com</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>Boston, MA</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>Capital partner for Oasis Apartments Cherry Creek (BMC Investments JV)</t>
+        </is>
+      </c>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/oasis-apartments-topping-out-299-milwaukee-cherry-creek</t>
+        </is>
+      </c>
+      <c r="G343" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H343" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I343" t="inlineStr"/>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>Kippah LLC</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr"/>
+      <c r="D344" t="inlineStr"/>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>Developer for 1415 Tremont Place adaptive reuse</t>
+        </is>
+      </c>
+      <c r="F344" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/tag/CBD</t>
+        </is>
+      </c>
+      <c r="G344" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H344" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I344" t="inlineStr"/>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>High Point Business Center LLC</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>Owner / Developer</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr"/>
+      <c r="D345" t="inlineStr"/>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>Owner entity for 192-unit affordable housing near DIA</t>
+        </is>
+      </c>
+      <c r="F345" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/192-unit-affordable-housing-high-point-denver</t>
+        </is>
+      </c>
+      <c r="G345" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H345" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I345" t="inlineStr"/>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>Brookfield Residential</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>Developer / Builder</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>https://www.brookfieldresidential.com</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>Calgary, Canada (Denver office)</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>Developer for Contour Townhomes at Central Park</t>
+        </is>
+      </c>
+      <c r="F346" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/brookfield-contour-townhomes-central-park-denver</t>
+        </is>
+      </c>
+      <c r="G346" t="inlineStr">
+        <is>
+          <t>developingmycity.com</t>
+        </is>
+      </c>
+      <c r="H346" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="I346" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -27302,7 +30135,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F146"/>
+  <dimension ref="A1:F166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -31985,6 +34818,646 @@
         </is>
       </c>
     </row>
+    <row r="147">
+      <c r="A147" s="3" t="inlineStr">
+        <is>
+          <t>Senior Housing Options Inc.</t>
+        </is>
+      </c>
+      <c r="B147" s="3" t="inlineStr">
+        <is>
+          <t>Barth Hotel Senior Housing</t>
+        </is>
+      </c>
+      <c r="C147" s="3" t="inlineStr">
+        <is>
+          <t>1514 17th Street, Denver</t>
+        </is>
+      </c>
+      <c r="D147" s="3" t="inlineStr">
+        <is>
+          <t>Senior Affordable Housing – 50 units (30-50% AMI), historic adaptive reuse</t>
+        </is>
+      </c>
+      <c r="E147" s="3" t="inlineStr">
+        <is>
+          <t>Concept Plan; $6M DDDA loan approved Jan 2026</t>
+        </is>
+      </c>
+      <c r="F147" s="3" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/barth-hotel-senior-housing-concept-1514-17th-denver</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>Eagle Propco 7 LLC</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>Holiday Inn Conversion – 240 Units</t>
+        </is>
+      </c>
+      <c r="C148" s="2" t="inlineStr">
+        <is>
+          <t>3333 N Quebec Street, Denver</t>
+        </is>
+      </c>
+      <c r="D148" s="2" t="inlineStr">
+        <is>
+          <t>Multifamily – 240 units, 11-story (hotel-to-residential)</t>
+        </is>
+      </c>
+      <c r="E148" s="2" t="inlineStr">
+        <is>
+          <t>Concept Plan Approved; advancing to SDP</t>
+        </is>
+      </c>
+      <c r="F148" s="2" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/holiday-inn-3333-n-quebec-240-unit-apartment-conversion-approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="3" t="inlineStr">
+        <is>
+          <t>Santa Fe Denver G LLC</t>
+        </is>
+      </c>
+      <c r="B149" s="3" t="inlineStr">
+        <is>
+          <t>Broadway Station Block 1</t>
+        </is>
+      </c>
+      <c r="C149" s="3" t="inlineStr">
+        <is>
+          <t>Broadway Station, South Denver</t>
+        </is>
+      </c>
+      <c r="D149" s="3" t="inlineStr">
+        <is>
+          <t>Multifamily – 367 units, 7-story + public plaza</t>
+        </is>
+      </c>
+      <c r="E149" s="3" t="inlineStr">
+        <is>
+          <t>SDP Review In Progress</t>
+        </is>
+      </c>
+      <c r="F149" s="3" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/7-story-residential-project-planned-for-broadway-station-block-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>ACE Padel</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>ACE Padel RiNo</t>
+        </is>
+      </c>
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>1812 35th Street, Denver</t>
+        </is>
+      </c>
+      <c r="D150" s="2" t="inlineStr">
+        <is>
+          <t>Sports / Recreation – 5 indoor + 3 outdoor padel courts + bar</t>
+        </is>
+      </c>
+      <c r="E150" s="2" t="inlineStr">
+        <is>
+          <t>Concept Plan Approved</t>
+        </is>
+      </c>
+      <c r="F150" s="2" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/ace-padel-rino-concept-plan-approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="3" t="inlineStr">
+        <is>
+          <t>Golub &amp; Company</t>
+        </is>
+      </c>
+      <c r="B151" s="3" t="inlineStr">
+        <is>
+          <t>Hopscotch Beer Garden – Denargo Market</t>
+        </is>
+      </c>
+      <c r="C151" s="3" t="inlineStr">
+        <is>
+          <t>3380 Denargo Street, Denver</t>
+        </is>
+      </c>
+      <c r="D151" s="3" t="inlineStr">
+        <is>
+          <t>Food &amp; Beverage / Entertainment – 17,000 SF outdoor beer garden</t>
+        </is>
+      </c>
+      <c r="E151" s="3" t="inlineStr">
+        <is>
+          <t>Approved; Opening late winter 2026</t>
+        </is>
+      </c>
+      <c r="F151" s="3" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/hopscotch-beer-garden-approved-for-denargo-market-opening-planned-for-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>Urban Green Development</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>Kensing LoHi Condos</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="inlineStr">
+        <is>
+          <t>1643 Boulder Street, Denver</t>
+        </is>
+      </c>
+      <c r="D152" s="2" t="inlineStr">
+        <is>
+          <t>For-Sale Condos – 35 units, 4-story</t>
+        </is>
+      </c>
+      <c r="E152" s="2" t="inlineStr">
+        <is>
+          <t>Nearing Completion / Grand Opening Jun 2026</t>
+        </is>
+      </c>
+      <c r="F152" s="2" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/kensing-lohi-condos-denver-lower-highlands</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="3" t="inlineStr">
+        <is>
+          <t>Colorado Coalition for the Homeless</t>
+        </is>
+      </c>
+      <c r="B153" s="3" t="inlineStr">
+        <is>
+          <t>Park Avenue Apartments – Globeville</t>
+        </is>
+      </c>
+      <c r="C153" s="3" t="inlineStr">
+        <is>
+          <t>3721 N Globeville Road, Denver</t>
+        </is>
+      </c>
+      <c r="D153" s="3" t="inlineStr">
+        <is>
+          <t>Supportive Housing – 60 units (La Quinta hotel adaptive reuse)</t>
+        </is>
+      </c>
+      <c r="E153" s="3" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
+      <c r="F153" s="3" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/park-avenue-apartments-globeville-supportive-housing</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>Denver Housing Authority</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>1139 Delaware – Supportive Housing</t>
+        </is>
+      </c>
+      <c r="C154" s="2" t="inlineStr">
+        <is>
+          <t>1139 Delaware Street, Denver</t>
+        </is>
+      </c>
+      <c r="D154" s="2" t="inlineStr">
+        <is>
+          <t>Supportive Housing – 80 units, 6-story</t>
+        </is>
+      </c>
+      <c r="E154" s="2" t="inlineStr">
+        <is>
+          <t>Under Review</t>
+        </is>
+      </c>
+      <c r="F154" s="2" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/1139-delaware-supportive-housing-renderings</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="3" t="inlineStr">
+        <is>
+          <t>RH Group</t>
+        </is>
+      </c>
+      <c r="B155" s="3" t="inlineStr">
+        <is>
+          <t>135-Unit Affordable Housing – 40th &amp; York</t>
+        </is>
+      </c>
+      <c r="C155" s="3" t="inlineStr">
+        <is>
+          <t>SE corner E 40th Ave &amp; York St, Denver</t>
+        </is>
+      </c>
+      <c r="D155" s="3" t="inlineStr">
+        <is>
+          <t>Affordable Housing – 135 units, 4-story, 100% income-restricted</t>
+        </is>
+      </c>
+      <c r="E155" s="3" t="inlineStr">
+        <is>
+          <t>Concept Plan (Intake in Progress)</t>
+        </is>
+      </c>
+      <c r="F155" s="3" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/40th-york-affordable-housing-concept-plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>Colorado Coalition for the Homeless</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>125-Unit Affordable Housing – North Federal</t>
+        </is>
+      </c>
+      <c r="C156" s="2" t="inlineStr">
+        <is>
+          <t>4745 N Federal Boulevard, Denver</t>
+        </is>
+      </c>
+      <c r="D156" s="2" t="inlineStr">
+        <is>
+          <t>Affordable + Supportive Housing – 125 units + daycare</t>
+        </is>
+      </c>
+      <c r="E156" s="2" t="inlineStr">
+        <is>
+          <t>Concept Review / Prop 123 Fast-Track</t>
+        </is>
+      </c>
+      <c r="F156" s="2" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/north-federal-affordable-housing-cch-rocky-mountain-lake</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="3" t="inlineStr">
+        <is>
+          <t>Denver Broncos</t>
+        </is>
+      </c>
+      <c r="B157" s="3" t="inlineStr">
+        <is>
+          <t>Burnham Yard Stadium</t>
+        </is>
+      </c>
+      <c r="C157" s="3" t="inlineStr">
+        <is>
+          <t>Burnham Yard, ~10th &amp; Osage, Denver</t>
+        </is>
+      </c>
+      <c r="D157" s="3" t="inlineStr">
+        <is>
+          <t>Stadium + Mixed-Use District – 150 acres</t>
+        </is>
+      </c>
+      <c r="E157" s="3" t="inlineStr">
+        <is>
+          <t>Rezoning / Early Planning</t>
+        </is>
+      </c>
+      <c r="F157" s="3" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/denver-broncos-burnham-yard-stadium-proposal-community-meeting</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>Kensington Development Partners</t>
+        </is>
+      </c>
+      <c r="B158" s="2" t="inlineStr">
+        <is>
+          <t>Link 56 – Parcel H Retail</t>
+        </is>
+      </c>
+      <c r="C158" s="2" t="inlineStr">
+        <is>
+          <t>E 56th Ave &amp; Tower Road, Denver (near DIA)</t>
+        </is>
+      </c>
+      <c r="D158" s="2" t="inlineStr">
+        <is>
+          <t>Retail – 2 buildings, 6,500 SF</t>
+        </is>
+      </c>
+      <c r="E158" s="2" t="inlineStr">
+        <is>
+          <t>Concept Plan / Design Revealed</t>
+        </is>
+      </c>
+      <c r="F158" s="2" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/link-56-parcel-h-retail-building-designs</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="3" t="inlineStr">
+        <is>
+          <t>Aaravya Investments</t>
+        </is>
+      </c>
+      <c r="B159" s="3" t="inlineStr">
+        <is>
+          <t>Elevate Travel Center – DIA</t>
+        </is>
+      </c>
+      <c r="C159" s="3" t="inlineStr">
+        <is>
+          <t>S of Peña Blvd, Denver</t>
+        </is>
+      </c>
+      <c r="D159" s="3" t="inlineStr">
+        <is>
+          <t>Travel Convenience Center – fueling, car wash, EV, retail</t>
+        </is>
+      </c>
+      <c r="E159" s="3" t="inlineStr">
+        <is>
+          <t>Under Construction; completion Summer 2026</t>
+        </is>
+      </c>
+      <c r="F159" s="3" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/elevate-travel-center-breaks-ground-near-denver-international-airport</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>Stillwater Capital</t>
+        </is>
+      </c>
+      <c r="B160" s="2" t="inlineStr">
+        <is>
+          <t>Four Seasons Private Residences – Cherry Creek</t>
+        </is>
+      </c>
+      <c r="C160" s="2" t="inlineStr">
+        <is>
+          <t>215-231 N Detroit Street, Denver</t>
+        </is>
+      </c>
+      <c r="D160" s="2" t="inlineStr">
+        <is>
+          <t>Luxury Condos – 41-42 units, 8-story</t>
+        </is>
+      </c>
+      <c r="E160" s="2" t="inlineStr">
+        <is>
+          <t>Urban Design Review (Jan 2026)</t>
+        </is>
+      </c>
+      <c r="F160" s="2" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/four-seasons-condos-cherry-creek-detroit-street</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="3" t="inlineStr">
+        <is>
+          <t>OliverBuchanan Group</t>
+        </is>
+      </c>
+      <c r="B161" s="3" t="inlineStr">
+        <is>
+          <t>Rock Drill RiNo Redevelopment</t>
+        </is>
+      </c>
+      <c r="C161" s="3" t="inlineStr">
+        <is>
+          <t>1717 E 39th Avenue, Denver</t>
+        </is>
+      </c>
+      <c r="D161" s="3" t="inlineStr">
+        <is>
+          <t>Mixed-Use – $585M (housing, retail, office, hotel on 6.7 acres)</t>
+        </is>
+      </c>
+      <c r="E161" s="3" t="inlineStr">
+        <is>
+          <t>Rezoning / TIF Financing Under Review</t>
+        </is>
+      </c>
+      <c r="F161" s="3" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/tag/Mixed-Use+Development</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>Continuum Partners</t>
+        </is>
+      </c>
+      <c r="B162" s="2" t="inlineStr">
+        <is>
+          <t>Historic Nurses Dorm – 9th+Colorado</t>
+        </is>
+      </c>
+      <c r="C162" s="2" t="inlineStr">
+        <is>
+          <t>4200 E 9th Avenue, Denver</t>
+        </is>
+      </c>
+      <c r="D162" s="2" t="inlineStr">
+        <is>
+          <t>Medical Office / Wellness / Coworking – 25,000-27,000 SF adaptive reuse</t>
+        </is>
+      </c>
+      <c r="E162" s="2" t="inlineStr">
+        <is>
+          <t>Concept Plan Filed</t>
+        </is>
+      </c>
+      <c r="F162" s="2" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/historic-nurses-dorm-9th-colorado-wellness-redevelopment</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="3" t="inlineStr">
+        <is>
+          <t>Buchanan Capital Partners</t>
+        </is>
+      </c>
+      <c r="B163" s="3" t="inlineStr">
+        <is>
+          <t>368-Unit Multifamily – South Havana</t>
+        </is>
+      </c>
+      <c r="C163" s="3" t="inlineStr">
+        <is>
+          <t>6901 S Havana Street, Centennial</t>
+        </is>
+      </c>
+      <c r="D163" s="3" t="inlineStr">
+        <is>
+          <t>Multifamily – 368 units, 14 buildings</t>
+        </is>
+      </c>
+      <c r="E163" s="3" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="F163" s="3" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/centennial-south-havana-multifamily-368-units</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
+        <is>
+          <t>City of Denver</t>
+        </is>
+      </c>
+      <c r="B164" s="2" t="inlineStr">
+        <is>
+          <t>Sloan's Lake Boathouse Renovation</t>
+        </is>
+      </c>
+      <c r="C164" s="2" t="inlineStr">
+        <is>
+          <t>Sloan's Lake Park, Denver</t>
+        </is>
+      </c>
+      <c r="D164" s="2" t="inlineStr">
+        <is>
+          <t>Recreation / Community Space – $7M renovation</t>
+        </is>
+      </c>
+      <c r="E164" s="2" t="inlineStr">
+        <is>
+          <t>Preferred Design Concept Released</t>
+        </is>
+      </c>
+      <c r="F164" s="2" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/sloans-lake-boathouse-renovation-preferred-design</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="3" t="inlineStr">
+        <is>
+          <t>National Western Center</t>
+        </is>
+      </c>
+      <c r="B165" s="3" t="inlineStr">
+        <is>
+          <t>National Western Center $185M Expansion</t>
+        </is>
+      </c>
+      <c r="C165" s="3" t="inlineStr">
+        <is>
+          <t>National Western Center campus, Denver</t>
+        </is>
+      </c>
+      <c r="D165" s="3" t="inlineStr">
+        <is>
+          <t>Equestrian Complex + 9-story Hotel + Parking – 726,000 SF, $185M</t>
+        </is>
+      </c>
+      <c r="E165" s="3" t="inlineStr">
+        <is>
+          <t>SDP Filed</t>
+        </is>
+      </c>
+      <c r="F165" s="3" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/national-western-center-185m-expansion</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="inlineStr">
+        <is>
+          <t>Brookfield Residential</t>
+        </is>
+      </c>
+      <c r="B166" s="2" t="inlineStr">
+        <is>
+          <t>Contour Townhomes – Central Park</t>
+        </is>
+      </c>
+      <c r="C166" s="2" t="inlineStr">
+        <is>
+          <t>E 47th Ave &amp; Beeler Court, Denver</t>
+        </is>
+      </c>
+      <c r="D166" s="2" t="inlineStr">
+        <is>
+          <t>Townhomes – 3-level, 2-3 BR</t>
+        </is>
+      </c>
+      <c r="E166" s="2" t="inlineStr">
+        <is>
+          <t>Under Construction / New Phase</t>
+        </is>
+      </c>
+      <c r="F166" s="2" t="inlineStr">
+        <is>
+          <t>https://www.developingmycity.com/denver/news/brookfield-contour-townhomes-central-park-denver</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:F120"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>